<commit_message>
Complete field RequestId WITH Automatic Form
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4FFA9F8-572A-4E04-BDC5-61F36664B614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188E5D2D-B460-4FE9-9109-D97700E755C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="22">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -63,96 +63,6 @@
   </si>
   <si>
     <t>Rejection reason</t>
-  </si>
-  <si>
-    <t>REQ-001</t>
-  </si>
-  <si>
-    <t>REQ-002</t>
-  </si>
-  <si>
-    <t>REQ-003</t>
-  </si>
-  <si>
-    <t>REQ-004</t>
-  </si>
-  <si>
-    <t>REQ-005</t>
-  </si>
-  <si>
-    <t>REQ-006</t>
-  </si>
-  <si>
-    <t>REQ-007</t>
-  </si>
-  <si>
-    <t>REQ-008</t>
-  </si>
-  <si>
-    <t>REQ-009</t>
-  </si>
-  <si>
-    <t>REQ-010</t>
-  </si>
-  <si>
-    <t>REQ-011</t>
-  </si>
-  <si>
-    <t>REQ-012</t>
-  </si>
-  <si>
-    <t>REQ-013</t>
-  </si>
-  <si>
-    <t>REQ-014</t>
-  </si>
-  <si>
-    <t>REQ-015</t>
-  </si>
-  <si>
-    <t>REQ-016</t>
-  </si>
-  <si>
-    <t>REQ-017</t>
-  </si>
-  <si>
-    <t>REQ-018</t>
-  </si>
-  <si>
-    <t>REQ-019</t>
-  </si>
-  <si>
-    <t>REQ-020</t>
-  </si>
-  <si>
-    <t>REQ-021</t>
-  </si>
-  <si>
-    <t>REQ-022</t>
-  </si>
-  <si>
-    <t>REQ-023</t>
-  </si>
-  <si>
-    <t>REQ-024</t>
-  </si>
-  <si>
-    <t>REQ-025</t>
-  </si>
-  <si>
-    <t>REQ-026</t>
-  </si>
-  <si>
-    <t>REQ-027</t>
-  </si>
-  <si>
-    <t>REQ-028</t>
-  </si>
-  <si>
-    <t>REQ-029</t>
-  </si>
-  <si>
-    <t>REQ-030</t>
   </si>
   <si>
     <t>Field Operations</t>
@@ -302,14 +212,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -328,7 +238,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -642,10 +552,58 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{14CAF9F0-18C4-4E4B-8E44-9F0250E5BB68}">
+  <we:reference id="wa200005502" version="1.0.0.11" store="es-ES" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200005502" version="1.0.0.11" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_GPT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CREATE_PROMPT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_LIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_HLIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CLASSIFY</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TRANSLATE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_EXTRACT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TAG</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CONVERT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_FORMAT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_SUMMARIZE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TABLE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_FILL</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_SPLIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_HSPLIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_EDIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_MATCH</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_VISION</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_WEB</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94A44B9A-1BC5-418D-8475-589934862B4F}">
   <dimension ref="A1:J33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -657,15 +615,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.2" x14ac:dyDescent="0.5">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -694,20 +652,21 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
+      <c r="A3" s="1" t="str">
+        <f>"REQ-"&amp;TEXT(ROW()-2,"000")</f>
+        <v>REQ-001</v>
       </c>
       <c r="B3" s="4">
         <v>46113</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1">
         <v>2</v>
@@ -715,20 +674,21 @@
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
+      <c r="A4" s="1" t="str">
+        <f t="shared" ref="A4:A33" si="0">"REQ-"&amp;TEXT(ROW()-2,"000")</f>
+        <v>REQ-002</v>
       </c>
       <c r="B4" s="4">
         <v>46114</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F4" s="1">
         <v>5</v>
@@ -736,20 +696,21 @@
       <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
+      <c r="A5" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-003</v>
       </c>
       <c r="B5" s="4">
         <v>46115</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F5" s="1">
         <v>6</v>
@@ -757,20 +718,21 @@
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
+      <c r="A6" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-004</v>
       </c>
       <c r="B6" s="4">
         <v>46116</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F6" s="1">
         <v>3</v>
@@ -778,20 +740,21 @@
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
+      <c r="A7" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-005</v>
       </c>
       <c r="B7" s="4">
         <v>46117</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F7" s="1">
         <v>5</v>
@@ -799,89 +762,93 @@
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
+      <c r="A8" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-006</v>
       </c>
       <c r="B8" s="4">
         <v>46118</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F8" s="1">
         <v>7</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>14</v>
+      <c r="A9" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-007</v>
       </c>
       <c r="B9" s="4">
         <v>46119</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F9" s="1">
         <v>12</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>15</v>
+      <c r="A10" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-008</v>
       </c>
       <c r="B10" s="4">
         <v>46120</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F10" s="1">
         <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
+      <c r="A11" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-009</v>
       </c>
       <c r="B11" s="4">
         <v>46121</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F11" s="1">
         <v>12</v>
@@ -889,87 +856,91 @@
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>17</v>
+      <c r="A12" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-010</v>
       </c>
       <c r="B12" s="4">
         <v>46122</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F12" s="1">
         <v>33</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>18</v>
+      <c r="A13" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-011</v>
       </c>
       <c r="B13" s="4">
         <v>46123</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F13" s="1">
         <v>20</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>19</v>
+      <c r="A14" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-012</v>
       </c>
       <c r="B14" s="4">
         <v>46124</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F14" s="1">
         <v>15</v>
       </c>
-      <c r="G14" s="8"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>20</v>
+      <c r="A15" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-013</v>
       </c>
       <c r="B15" s="4">
         <v>46125</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F15" s="1">
         <v>16</v>
@@ -977,20 +948,21 @@
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>21</v>
+      <c r="A16" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-014</v>
       </c>
       <c r="B16" s="4">
         <v>46126</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F16" s="1">
         <v>17</v>
@@ -998,20 +970,21 @@
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>22</v>
+      <c r="A17" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-015</v>
       </c>
       <c r="B17" s="4">
         <v>46127</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F17" s="1">
         <v>12</v>
@@ -1019,20 +992,21 @@
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>23</v>
+      <c r="A18" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-016</v>
       </c>
       <c r="B18" s="4">
         <v>46128</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F18" s="1">
         <v>23</v>
@@ -1040,20 +1014,21 @@
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>24</v>
+      <c r="A19" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-017</v>
       </c>
       <c r="B19" s="4">
         <v>46129</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F19" s="1">
         <v>15</v>
@@ -1061,20 +1036,21 @@
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>25</v>
+      <c r="A20" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-018</v>
       </c>
       <c r="B20" s="4">
         <v>46130</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F20" s="1">
         <v>16</v>
@@ -1082,20 +1058,21 @@
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>26</v>
+      <c r="A21" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-019</v>
       </c>
       <c r="B21" s="4">
         <v>46131</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F21" s="1">
         <v>19</v>
@@ -1103,20 +1080,21 @@
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>27</v>
+      <c r="A22" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-020</v>
       </c>
       <c r="B22" s="4">
         <v>46132</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F22" s="1">
         <v>18</v>
@@ -1124,20 +1102,21 @@
       <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>28</v>
+      <c r="A23" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-021</v>
       </c>
       <c r="B23" s="4">
         <v>46133</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F23" s="1">
         <v>20</v>
@@ -1145,20 +1124,21 @@
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>29</v>
+      <c r="A24" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-022</v>
       </c>
       <c r="B24" s="4">
         <v>46134</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F24" s="1">
         <v>24</v>
@@ -1166,20 +1146,21 @@
       <c r="G24" s="1"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>30</v>
+      <c r="A25" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-023</v>
       </c>
       <c r="B25" s="4">
         <v>46135</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F25" s="1">
         <v>26</v>
@@ -1187,20 +1168,21 @@
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>31</v>
+      <c r="A26" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-024</v>
       </c>
       <c r="B26" s="4">
         <v>46136</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F26" s="1">
         <v>28</v>
@@ -1208,20 +1190,21 @@
       <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>32</v>
+      <c r="A27" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-025</v>
       </c>
       <c r="B27" s="4">
         <v>46137</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F27" s="1">
         <v>29</v>
@@ -1229,20 +1212,21 @@
       <c r="G27" s="1"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>33</v>
+      <c r="A28" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-026</v>
       </c>
       <c r="B28" s="4">
         <v>46138</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F28" s="1">
         <v>31</v>
@@ -1250,20 +1234,21 @@
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>34</v>
+      <c r="A29" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-027</v>
       </c>
       <c r="B29" s="4">
         <v>46139</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F29" s="1">
         <v>13</v>
@@ -1271,20 +1256,21 @@
       <c r="G29" s="1"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>35</v>
+      <c r="A30" s="1" t="str">
+        <f>"REQ-"&amp;TEXT(ROW()-2,"000")</f>
+        <v>REQ-028</v>
       </c>
       <c r="B30" s="4">
         <v>46140</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F30" s="1">
         <v>12</v>
@@ -1292,20 +1278,21 @@
       <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>36</v>
+      <c r="A31" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-029</v>
       </c>
       <c r="B31" s="4">
         <v>46141</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F31" s="1">
         <v>10</v>
@@ -1313,28 +1300,33 @@
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>37</v>
+      <c r="A32" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-030</v>
       </c>
       <c r="B32" s="4">
         <v>46142</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F32" s="1">
         <v>27</v>
       </c>
       <c r="G32" s="1"/>
     </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D33" s="7"/>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>REQ-031</v>
+      </c>
+      <c r="D33" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
complete field DATE WITH excel formula
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188E5D2D-B460-4FE9-9109-D97700E755C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECB9867-BD22-4E56-A097-1F1D95412C33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -155,7 +155,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -202,11 +202,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -220,6 +233,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -657,7 +672,8 @@
         <v>REQ-001</v>
       </c>
       <c r="B3" s="4">
-        <v>46113</v>
+        <f ca="1">DATE(2026,4,1)+INT(RAND()*59)</f>
+        <v>46171</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>8</v>
@@ -679,7 +695,8 @@
         <v>REQ-002</v>
       </c>
       <c r="B4" s="4">
-        <v>46114</v>
+        <f t="shared" ref="B4:B32" ca="1" si="1">DATE(2026,4,1)+INT(RAND()*59)</f>
+        <v>46121</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>9</v>
@@ -701,7 +718,8 @@
         <v>REQ-003</v>
       </c>
       <c r="B5" s="4">
-        <v>46115</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46151</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>10</v>
@@ -723,7 +741,8 @@
         <v>REQ-004</v>
       </c>
       <c r="B6" s="4">
-        <v>46116</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46117</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
@@ -745,7 +764,8 @@
         <v>REQ-005</v>
       </c>
       <c r="B7" s="4">
-        <v>46117</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46113</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>11</v>
@@ -767,7 +787,8 @@
         <v>REQ-006</v>
       </c>
       <c r="B8" s="4">
-        <v>46118</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46113</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>11</v>
@@ -791,7 +812,8 @@
         <v>REQ-007</v>
       </c>
       <c r="B9" s="4">
-        <v>46119</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46146</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>11</v>
@@ -815,7 +837,8 @@
         <v>REQ-008</v>
       </c>
       <c r="B10" s="4">
-        <v>46120</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46146</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>11</v>
@@ -839,7 +862,8 @@
         <v>REQ-009</v>
       </c>
       <c r="B11" s="4">
-        <v>46121</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46166</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>9</v>
@@ -861,7 +885,8 @@
         <v>REQ-010</v>
       </c>
       <c r="B12" s="4">
-        <v>46122</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46170</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>8</v>
@@ -885,7 +910,8 @@
         <v>REQ-011</v>
       </c>
       <c r="B13" s="4">
-        <v>46123</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46137</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>10</v>
@@ -909,7 +935,8 @@
         <v>REQ-012</v>
       </c>
       <c r="B14" s="4">
-        <v>46124</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46119</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>8</v>
@@ -931,7 +958,8 @@
         <v>REQ-013</v>
       </c>
       <c r="B15" s="4">
-        <v>46125</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46142</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>9</v>
@@ -953,7 +981,8 @@
         <v>REQ-014</v>
       </c>
       <c r="B16" s="4">
-        <v>46126</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46144</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>11</v>
@@ -975,7 +1004,8 @@
         <v>REQ-015</v>
       </c>
       <c r="B17" s="4">
-        <v>46127</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46132</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>11</v>
@@ -997,7 +1027,8 @@
         <v>REQ-016</v>
       </c>
       <c r="B18" s="4">
-        <v>46128</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46120</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>10</v>
@@ -1019,7 +1050,8 @@
         <v>REQ-017</v>
       </c>
       <c r="B19" s="4">
-        <v>46129</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46121</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>10</v>
@@ -1041,7 +1073,8 @@
         <v>REQ-018</v>
       </c>
       <c r="B20" s="4">
-        <v>46130</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46133</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>9</v>
@@ -1063,7 +1096,8 @@
         <v>REQ-019</v>
       </c>
       <c r="B21" s="4">
-        <v>46131</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46137</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>9</v>
@@ -1085,7 +1119,8 @@
         <v>REQ-020</v>
       </c>
       <c r="B22" s="4">
-        <v>46132</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46135</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>11</v>
@@ -1107,7 +1142,8 @@
         <v>REQ-021</v>
       </c>
       <c r="B23" s="4">
-        <v>46133</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46141</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>11</v>
@@ -1129,7 +1165,8 @@
         <v>REQ-022</v>
       </c>
       <c r="B24" s="4">
-        <v>46134</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46162</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>8</v>
@@ -1151,7 +1188,8 @@
         <v>REQ-023</v>
       </c>
       <c r="B25" s="4">
-        <v>46135</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46158</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>8</v>
@@ -1173,7 +1211,8 @@
         <v>REQ-024</v>
       </c>
       <c r="B26" s="4">
-        <v>46136</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46168</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>8</v>
@@ -1195,7 +1234,8 @@
         <v>REQ-025</v>
       </c>
       <c r="B27" s="4">
-        <v>46137</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46147</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>8</v>
@@ -1217,7 +1257,8 @@
         <v>REQ-026</v>
       </c>
       <c r="B28" s="4">
-        <v>46138</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46144</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>10</v>
@@ -1239,7 +1280,8 @@
         <v>REQ-027</v>
       </c>
       <c r="B29" s="4">
-        <v>46139</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46114</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>9</v>
@@ -1261,7 +1303,8 @@
         <v>REQ-028</v>
       </c>
       <c r="B30" s="4">
-        <v>46140</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46154</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>9</v>
@@ -1283,7 +1326,8 @@
         <v>REQ-029</v>
       </c>
       <c r="B31" s="4">
-        <v>46141</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46120</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>9</v>
@@ -1300,12 +1344,13 @@
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="str">
+      <c r="A32" s="9" t="str">
         <f t="shared" si="0"/>
         <v>REQ-030</v>
       </c>
       <c r="B32" s="4">
-        <v>46142</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46148</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>10</v>
@@ -1322,10 +1367,7 @@
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>REQ-031</v>
-      </c>
+      <c r="A33" s="10"/>
       <c r="D33" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
complete field area with excel formula
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BECB9867-BD22-4E56-A097-1F1D95412C33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42BC053C-54BA-40AB-A37A-B5AD856435CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="18">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -63,18 +63,6 @@
   </si>
   <si>
     <t>Rejection reason</t>
-  </si>
-  <si>
-    <t>Field Operations</t>
-  </si>
-  <si>
-    <t>Packaging</t>
-  </si>
-  <si>
-    <t>Administration</t>
-  </si>
-  <si>
-    <t>Logistics</t>
   </si>
   <si>
     <t>Materials</t>
@@ -155,7 +143,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -202,24 +190,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -233,7 +208,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -673,16 +647,17 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46171</v>
-      </c>
-      <c r="C3" s="1" t="s">
+        <v>46155</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
+        <v>Logistics</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F3" s="1">
         <v>2</v>
@@ -696,16 +671,17 @@
       </c>
       <c r="B4" s="4">
         <f t="shared" ref="B4:B32" ca="1" si="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46121</v>
-      </c>
-      <c r="C4" s="1" t="s">
+        <v>46141</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <f t="shared" ref="C4:C32" ca="1" si="2">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
+        <v>Field opetations</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E4" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F4" s="1">
         <v>5</v>
@@ -719,16 +695,17 @@
       </c>
       <c r="B5" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46151</v>
-      </c>
-      <c r="C5" s="1" t="s">
+        <v>46140</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Logistics</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1">
         <v>6</v>
@@ -742,16 +719,17 @@
       </c>
       <c r="B6" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46117</v>
-      </c>
-      <c r="C6" s="1" t="s">
+        <v>46126</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F6" s="1">
         <v>3</v>
@@ -765,16 +743,17 @@
       </c>
       <c r="B7" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46113</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>46141</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F7" s="1">
         <v>5</v>
@@ -788,22 +767,23 @@
       </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46113</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>11</v>
+        <v>46129</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F8" s="1">
         <v>7</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -813,22 +793,23 @@
       </c>
       <c r="B9" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46146</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>11</v>
+        <v>46128</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F9" s="1">
         <v>12</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -838,22 +819,23 @@
       </c>
       <c r="B10" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46146</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>11</v>
+        <v>46158</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Logistics</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="F10" s="1">
         <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -863,16 +845,17 @@
       </c>
       <c r="B11" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46166</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>9</v>
+        <v>46113</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F11" s="1">
         <v>12</v>
@@ -886,22 +869,23 @@
       </c>
       <c r="B12" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46170</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>8</v>
+        <v>46116</v>
+      </c>
+      <c r="C12" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Logistics</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F12" s="1">
         <v>33</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -911,22 +895,23 @@
       </c>
       <c r="B13" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46137</v>
-      </c>
-      <c r="C13" s="1" t="s">
+        <v>46151</v>
+      </c>
+      <c r="C13" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Logistics</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="E13" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F13" s="1">
         <v>20</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -936,16 +921,17 @@
       </c>
       <c r="B14" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46119</v>
-      </c>
-      <c r="C14" s="1" t="s">
+        <v>46131</v>
+      </c>
+      <c r="C14" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="E14" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F14" s="1">
         <v>15</v>
@@ -959,16 +945,17 @@
       </c>
       <c r="B15" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46142</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>9</v>
+        <v>46132</v>
+      </c>
+      <c r="C15" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Field opetations</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F15" s="1">
         <v>16</v>
@@ -982,16 +969,17 @@
       </c>
       <c r="B16" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46144</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>11</v>
+        <v>46132</v>
+      </c>
+      <c r="C16" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F16" s="1">
         <v>17</v>
@@ -1005,16 +993,17 @@
       </c>
       <c r="B17" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46132</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>11</v>
+        <v>46149</v>
+      </c>
+      <c r="C17" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F17" s="1">
         <v>12</v>
@@ -1028,16 +1017,17 @@
       </c>
       <c r="B18" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46120</v>
-      </c>
-      <c r="C18" s="1" t="s">
+        <v>46158</v>
+      </c>
+      <c r="C18" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="E18" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F18" s="1">
         <v>23</v>
@@ -1051,16 +1041,17 @@
       </c>
       <c r="B19" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46121</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>10</v>
+        <v>46164</v>
+      </c>
+      <c r="C19" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F19" s="1">
         <v>15</v>
@@ -1074,16 +1065,17 @@
       </c>
       <c r="B20" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46133</v>
-      </c>
-      <c r="C20" s="1" t="s">
+        <v>46117</v>
+      </c>
+      <c r="C20" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Field opetations</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="F20" s="1">
         <v>16</v>
@@ -1097,16 +1089,17 @@
       </c>
       <c r="B21" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46137</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>9</v>
+        <v>46136</v>
+      </c>
+      <c r="C21" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F21" s="1">
         <v>19</v>
@@ -1120,16 +1113,17 @@
       </c>
       <c r="B22" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46135</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>11</v>
+        <v>46152</v>
+      </c>
+      <c r="C22" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F22" s="1">
         <v>18</v>
@@ -1143,16 +1137,17 @@
       </c>
       <c r="B23" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46141</v>
-      </c>
-      <c r="C23" s="1" t="s">
+        <v>46166</v>
+      </c>
+      <c r="C23" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Field opetations</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="E23" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F23" s="1">
         <v>20</v>
@@ -1166,16 +1161,17 @@
       </c>
       <c r="B24" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46162</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>8</v>
+        <v>46127</v>
+      </c>
+      <c r="C24" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Field opetations</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F24" s="1">
         <v>24</v>
@@ -1189,16 +1185,17 @@
       </c>
       <c r="B25" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46158</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>8</v>
+        <v>46139</v>
+      </c>
+      <c r="C25" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Logistics</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F25" s="1">
         <v>26</v>
@@ -1212,16 +1209,17 @@
       </c>
       <c r="B26" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46168</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>8</v>
+        <v>46159</v>
+      </c>
+      <c r="C26" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Field opetations</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F26" s="1">
         <v>28</v>
@@ -1235,16 +1233,17 @@
       </c>
       <c r="B27" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46147</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>8</v>
+        <v>46153</v>
+      </c>
+      <c r="C27" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="F27" s="1">
         <v>29</v>
@@ -1258,16 +1257,17 @@
       </c>
       <c r="B28" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46144</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>10</v>
+        <v>46117</v>
+      </c>
+      <c r="C28" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Packaging</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F28" s="1">
         <v>31</v>
@@ -1281,16 +1281,17 @@
       </c>
       <c r="B29" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46114</v>
-      </c>
-      <c r="C29" s="1" t="s">
+        <v>46120</v>
+      </c>
+      <c r="C29" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E29" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F29" s="1">
         <v>13</v>
@@ -1304,16 +1305,17 @@
       </c>
       <c r="B30" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46154</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>9</v>
+        <v>46163</v>
+      </c>
+      <c r="C30" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Administration</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F30" s="1">
         <v>12</v>
@@ -1327,16 +1329,17 @@
       </c>
       <c r="B31" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46120</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>9</v>
+        <v>46166</v>
+      </c>
+      <c r="C31" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Field opetations</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F31" s="1">
         <v>10</v>
@@ -1344,22 +1347,23 @@
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="str">
+      <c r="A32" s="1" t="str">
         <f t="shared" si="0"/>
         <v>REQ-030</v>
       </c>
       <c r="B32" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46148</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>10</v>
+        <v>46147</v>
+      </c>
+      <c r="C32" s="1" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>Logistics</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F32" s="1">
         <v>27</v>
@@ -1367,7 +1371,7 @@
       <c r="G32" s="1"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
+      <c r="A33" s="9"/>
       <c r="D33" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
complete field request type with excel formula
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42BC053C-54BA-40AB-A37A-B5AD856435CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2CB6FE-1ECA-44A7-82C6-D009D9A87D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="14">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -63,18 +63,6 @@
   </si>
   <si>
     <t>Rejection reason</t>
-  </si>
-  <si>
-    <t>Materials</t>
-  </si>
-  <si>
-    <t>Personnel</t>
-  </si>
-  <si>
-    <t>Equipment</t>
-  </si>
-  <si>
-    <t>Supplies</t>
   </si>
   <si>
     <t>Approved</t>
@@ -647,17 +635,18 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46155</v>
+        <v>46141</v>
       </c>
       <c r="C3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
-        <v>Logistics</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
+        <v>Field opetations</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
+        <v>Perssonel</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F3" s="1">
         <v>2</v>
@@ -671,17 +660,18 @@
       </c>
       <c r="B4" s="4">
         <f t="shared" ref="B4:B32" ca="1" si="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46141</v>
+        <v>46137</v>
       </c>
       <c r="C4" s="1" t="str">
         <f t="shared" ref="C4:C32" ca="1" si="2">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
         <v>Field opetations</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>9</v>
+      <c r="D4" s="1" t="str">
+        <f t="shared" ref="D4:D32" ca="1" si="3">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
+        <v>Perssonel</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F4" s="1">
         <v>5</v>
@@ -695,17 +685,18 @@
       </c>
       <c r="B5" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46140</v>
+        <v>46120</v>
       </c>
       <c r="C5" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>Field opetations</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Materials</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F5" s="1">
         <v>6</v>
@@ -719,17 +710,18 @@
       </c>
       <c r="B6" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46126</v>
+        <v>46114</v>
       </c>
       <c r="C6" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>Administration</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Materials</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F6" s="1">
         <v>3</v>
@@ -743,17 +735,18 @@
       </c>
       <c r="B7" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46141</v>
+        <v>46159</v>
       </c>
       <c r="C7" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>Administration</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F7" s="1">
         <v>5</v>
@@ -767,23 +760,24 @@
       </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46129</v>
+        <v>46156</v>
       </c>
       <c r="C8" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>8</v>
+        <v>Packaging</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F8" s="1">
         <v>7</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -793,23 +787,24 @@
       </c>
       <c r="B9" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46128</v>
+        <v>46116</v>
       </c>
       <c r="C9" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>8</v>
+        <v>Field opetations</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Materials</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F9" s="1">
         <v>12</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -819,23 +814,24 @@
       </c>
       <c r="B10" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46158</v>
+        <v>46119</v>
       </c>
       <c r="C10" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
-      </c>
-      <c r="D10" s="1" t="s">
+        <v>Field opetations</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F10" s="1">
         <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -845,17 +841,18 @@
       </c>
       <c r="B11" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46113</v>
+        <v>46153</v>
       </c>
       <c r="C11" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>11</v>
+        <v>Logistics</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F11" s="1">
         <v>12</v>
@@ -869,23 +866,24 @@
       </c>
       <c r="B12" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46116</v>
+        <v>46169</v>
       </c>
       <c r="C12" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>11</v>
+        <v>Field opetations</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F12" s="1">
         <v>33</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -895,23 +893,24 @@
       </c>
       <c r="B13" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46151</v>
+        <v>46164</v>
       </c>
       <c r="C13" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>10</v>
+        <v>Field opetations</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Perssonel</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F13" s="1">
         <v>20</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -921,17 +920,18 @@
       </c>
       <c r="B14" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46131</v>
+        <v>46165</v>
       </c>
       <c r="C14" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>8</v>
+        <v>Logistics</v>
+      </c>
+      <c r="D14" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F14" s="1">
         <v>15</v>
@@ -945,17 +945,18 @@
       </c>
       <c r="B15" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46132</v>
+        <v>46162</v>
       </c>
       <c r="C15" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
         <v>Field opetations</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>8</v>
+      <c r="D15" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F15" s="1">
         <v>16</v>
@@ -969,17 +970,18 @@
       </c>
       <c r="B16" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46132</v>
+        <v>46169</v>
       </c>
       <c r="C16" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
         <v>Administration</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>10</v>
+      <c r="D16" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Perssonel</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F16" s="1">
         <v>17</v>
@@ -993,17 +995,18 @@
       </c>
       <c r="B17" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46149</v>
+        <v>46137</v>
       </c>
       <c r="C17" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>10</v>
+        <v>Field opetations</v>
+      </c>
+      <c r="D17" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F17" s="1">
         <v>12</v>
@@ -1017,17 +1020,18 @@
       </c>
       <c r="B18" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46158</v>
+        <v>46130</v>
       </c>
       <c r="C18" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>10</v>
+        <v>Packaging</v>
+      </c>
+      <c r="D18" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Perssonel</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F18" s="1">
         <v>23</v>
@@ -1041,17 +1045,18 @@
       </c>
       <c r="B19" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="C19" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
         <v>Packaging</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>9</v>
+      <c r="D19" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Materials</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F19" s="1">
         <v>15</v>
@@ -1065,17 +1070,18 @@
       </c>
       <c r="B20" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46117</v>
+        <v>46154</v>
       </c>
       <c r="C20" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
-      </c>
-      <c r="D20" s="1" t="s">
+        <v>Packaging</v>
+      </c>
+      <c r="D20" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F20" s="1">
         <v>16</v>
@@ -1089,17 +1095,18 @@
       </c>
       <c r="B21" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46136</v>
+        <v>46123</v>
       </c>
       <c r="C21" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
         <v>Administration</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>10</v>
+      <c r="D21" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F21" s="1">
         <v>19</v>
@@ -1113,17 +1120,18 @@
       </c>
       <c r="B22" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46152</v>
+        <v>46139</v>
       </c>
       <c r="C22" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>10</v>
+        <v>Administration</v>
+      </c>
+      <c r="D22" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Materials</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F22" s="1">
         <v>18</v>
@@ -1137,17 +1145,18 @@
       </c>
       <c r="B23" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46166</v>
+        <v>46143</v>
       </c>
       <c r="C23" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>11</v>
+        <v>Logistics</v>
+      </c>
+      <c r="D23" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F23" s="1">
         <v>20</v>
@@ -1161,17 +1170,18 @@
       </c>
       <c r="B24" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46127</v>
+        <v>46169</v>
       </c>
       <c r="C24" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
         <v>Field opetations</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>11</v>
+      <c r="D24" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F24" s="1">
         <v>24</v>
@@ -1185,17 +1195,18 @@
       </c>
       <c r="B25" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46133</v>
       </c>
       <c r="C25" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
         <v>Logistics</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>11</v>
+      <c r="D25" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F25" s="1">
         <v>26</v>
@@ -1209,17 +1220,18 @@
       </c>
       <c r="B26" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46159</v>
+        <v>46115</v>
       </c>
       <c r="C26" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>11</v>
+        <v>Packaging</v>
+      </c>
+      <c r="D26" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F26" s="1">
         <v>28</v>
@@ -1233,17 +1245,18 @@
       </c>
       <c r="B27" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46153</v>
+        <v>46164</v>
       </c>
       <c r="C27" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
         <v>Packaging</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Perssonel</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F27" s="1">
         <v>29</v>
@@ -1257,17 +1270,18 @@
       </c>
       <c r="B28" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46117</v>
+        <v>46149</v>
       </c>
       <c r="C28" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>Logistics</v>
+      </c>
+      <c r="D28" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Perssonel</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F28" s="1">
         <v>31</v>
@@ -1281,17 +1295,18 @@
       </c>
       <c r="B29" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46120</v>
+        <v>46128</v>
       </c>
       <c r="C29" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>9</v>
+        <v>Packaging</v>
+      </c>
+      <c r="D29" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F29" s="1">
         <v>13</v>
@@ -1305,17 +1320,18 @@
       </c>
       <c r="B30" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46163</v>
+        <v>46166</v>
       </c>
       <c r="C30" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>8</v>
+        <v>Packaging</v>
+      </c>
+      <c r="D30" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Equipment</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F30" s="1">
         <v>12</v>
@@ -1329,17 +1345,18 @@
       </c>
       <c r="B31" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46166</v>
+        <v>46161</v>
       </c>
       <c r="C31" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>8</v>
+        <v>Packaging</v>
+      </c>
+      <c r="D31" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F31" s="1">
         <v>10</v>
@@ -1353,17 +1370,18 @@
       </c>
       <c r="B32" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46147</v>
+        <v>46118</v>
       </c>
       <c r="C32" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>9</v>
+        <v>Administration</v>
+      </c>
+      <c r="D32" s="1" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>Supplies</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F32" s="1">
         <v>27</v>

</xml_diff>

<commit_message>
complete field status and response time with excel formula
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2CB6FE-1ECA-44A7-82C6-D009D9A87D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E40C24-8FA5-4A73-874C-907A54DD6A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -63,12 +63,6 @@
   </si>
   <si>
     <t>Rejection reason</t>
-  </si>
-  <si>
-    <t>Approved</t>
-  </si>
-  <si>
-    <t>Reject</t>
   </si>
   <si>
     <t>Bugget Exceeded</t>
@@ -182,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -196,7 +190,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -635,46 +628,50 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46141</v>
+        <v>46155</v>
       </c>
       <c r="C3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
-        <v>Perssonel</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>Materials</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <f ca="1">IF(RAND()&lt;0.7,"Approved","Reject")</f>
+        <v>Reject</v>
       </c>
       <c r="F3" s="1">
-        <v>2</v>
+        <f ca="1">RANDBETWEEN(4,48)</f>
+        <v>20</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="str">
-        <f t="shared" ref="A4:A33" si="0">"REQ-"&amp;TEXT(ROW()-2,"000")</f>
+        <f t="shared" ref="A4:A32" si="0">"REQ-"&amp;TEXT(ROW()-2,"000")</f>
         <v>REQ-002</v>
       </c>
       <c r="B4" s="4">
         <f t="shared" ref="B4:B32" ca="1" si="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46137</v>
+        <v>46162</v>
       </c>
       <c r="C4" s="1" t="str">
         <f t="shared" ref="C4:C32" ca="1" si="2">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D4" s="1" t="str">
         <f t="shared" ref="D4:D32" ca="1" si="3">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
-        <v>Perssonel</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
+        <v>Equipment</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <f t="shared" ref="E4:E32" ca="1" si="4">IF(RAND()&lt;0.7,"Approved","Reject")</f>
+        <v>Approved</v>
       </c>
       <c r="F4" s="1">
-        <v>5</v>
+        <f t="shared" ref="F4:F32" ca="1" si="5">RANDBETWEEN(4,48)</f>
+        <v>32</v>
       </c>
       <c r="G4" s="1"/>
     </row>
@@ -685,21 +682,23 @@
       </c>
       <c r="B5" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46120</v>
+        <v>46122</v>
       </c>
       <c r="C5" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Packaging</v>
       </c>
       <c r="D5" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>8</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F5" s="1">
-        <v>6</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>23</v>
       </c>
       <c r="G5" s="1"/>
     </row>
@@ -710,21 +709,23 @@
       </c>
       <c r="B6" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46114</v>
+        <v>46143</v>
       </c>
       <c r="C6" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Field opetations</v>
       </c>
       <c r="D6" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>8</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F6" s="1">
-        <v>3</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>41</v>
       </c>
       <c r="G6" s="1"/>
     </row>
@@ -735,20 +736,22 @@
       </c>
       <c r="B7" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46159</v>
+        <v>46130</v>
       </c>
       <c r="C7" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D7" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>Supplies</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>8</v>
+      <c r="E7" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F7" s="1">
+        <f t="shared" ca="1" si="5"/>
         <v>5</v>
       </c>
       <c r="G7" s="1"/>
@@ -760,7 +763,7 @@
       </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46156</v>
+        <v>46124</v>
       </c>
       <c r="C8" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -768,16 +771,18 @@
       </c>
       <c r="D8" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>9</v>
+        <v>Materials</v>
+      </c>
+      <c r="E8" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F8" s="1">
-        <v>7</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>10</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -787,24 +792,26 @@
       </c>
       <c r="B9" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46116</v>
+        <v>46121</v>
       </c>
       <c r="C9" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Packaging</v>
       </c>
       <c r="D9" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>Materials</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" ca="1" si="5"/>
+        <v>25</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="F9" s="1">
-        <v>12</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -814,7 +821,7 @@
       </c>
       <c r="B10" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46119</v>
+        <v>46128</v>
       </c>
       <c r="C10" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -822,16 +829,18 @@
       </c>
       <c r="D10" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>9</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E10" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F10" s="1">
-        <v>23</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>26</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -841,7 +850,7 @@
       </c>
       <c r="B11" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46153</v>
+        <v>46157</v>
       </c>
       <c r="C11" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -849,13 +858,15 @@
       </c>
       <c r="D11" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>8</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E11" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F11" s="1">
-        <v>12</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>44</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -866,24 +877,26 @@
       </c>
       <c r="B12" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46169</v>
+        <v>46145</v>
       </c>
       <c r="C12" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D12" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>9</v>
+        <v>Equipment</v>
+      </c>
+      <c r="E12" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F12" s="1">
-        <v>33</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>16</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -893,24 +906,26 @@
       </c>
       <c r="B13" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46164</v>
+        <v>46161</v>
       </c>
       <c r="C13" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Administration</v>
       </c>
       <c r="D13" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>Perssonel</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>9</v>
+      <c r="E13" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F13" s="1">
-        <v>20</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>24</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -920,21 +935,23 @@
       </c>
       <c r="B14" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46165</v>
+        <v>46162</v>
       </c>
       <c r="C14" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Packaging</v>
       </c>
       <c r="D14" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>9</v>
+        <v>Equipment</v>
+      </c>
+      <c r="E14" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F14" s="1">
-        <v>15</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>39</v>
       </c>
       <c r="G14" s="6"/>
     </row>
@@ -945,7 +962,7 @@
       </c>
       <c r="B15" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46162</v>
+        <v>46158</v>
       </c>
       <c r="C15" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -955,11 +972,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>Equipment</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>8</v>
+      <c r="E15" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F15" s="1">
-        <v>16</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>9</v>
       </c>
       <c r="G15" s="1"/>
     </row>
@@ -970,21 +989,23 @@
       </c>
       <c r="B16" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46169</v>
+        <v>46146</v>
       </c>
       <c r="C16" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Logistics</v>
       </c>
       <c r="D16" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>8</v>
+        <v>Materials</v>
+      </c>
+      <c r="E16" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F16" s="1">
-        <v>17</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>47</v>
       </c>
       <c r="G16" s="1"/>
     </row>
@@ -995,21 +1016,23 @@
       </c>
       <c r="B17" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="C17" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D17" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>8</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E17" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F17" s="1">
-        <v>12</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>9</v>
       </c>
       <c r="G17" s="1"/>
     </row>
@@ -1020,21 +1043,23 @@
       </c>
       <c r="B18" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46130</v>
+        <v>46147</v>
       </c>
       <c r="C18" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D18" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>9</v>
+        <v>Equipment</v>
+      </c>
+      <c r="E18" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F18" s="1">
-        <v>23</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>6</v>
       </c>
       <c r="G18" s="1"/>
     </row>
@@ -1045,7 +1070,7 @@
       </c>
       <c r="B19" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46165</v>
+        <v>46126</v>
       </c>
       <c r="C19" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1055,11 +1080,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>Materials</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>8</v>
+      <c r="E19" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F19" s="1">
-        <v>15</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>44</v>
       </c>
       <c r="G19" s="1"/>
     </row>
@@ -1070,21 +1097,23 @@
       </c>
       <c r="B20" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46154</v>
+        <v>46118</v>
       </c>
       <c r="C20" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D20" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>9</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E20" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F20" s="1">
-        <v>16</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>28</v>
       </c>
       <c r="G20" s="1"/>
     </row>
@@ -1095,21 +1124,23 @@
       </c>
       <c r="B21" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46123</v>
+        <v>46124</v>
       </c>
       <c r="C21" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D21" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>Equipment</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>8</v>
+      <c r="E21" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F21" s="1">
-        <v>19</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>29</v>
       </c>
       <c r="G21" s="1"/>
     </row>
@@ -1120,21 +1151,23 @@
       </c>
       <c r="B22" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="C22" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D22" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>8</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E22" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F22" s="1">
-        <v>18</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>17</v>
       </c>
       <c r="G22" s="1"/>
     </row>
@@ -1145,7 +1178,7 @@
       </c>
       <c r="B23" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46143</v>
+        <v>46141</v>
       </c>
       <c r="C23" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1153,13 +1186,15 @@
       </c>
       <c r="D23" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>8</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E23" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F23" s="1">
-        <v>20</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>35</v>
       </c>
       <c r="G23" s="1"/>
     </row>
@@ -1170,21 +1205,23 @@
       </c>
       <c r="B24" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46169</v>
+        <v>46124</v>
       </c>
       <c r="C24" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Administration</v>
       </c>
       <c r="D24" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>8</v>
+        <v>Equipment</v>
+      </c>
+      <c r="E24" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F24" s="1">
-        <v>24</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>32</v>
       </c>
       <c r="G24" s="1"/>
     </row>
@@ -1195,21 +1232,23 @@
       </c>
       <c r="B25" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46133</v>
+        <v>46145</v>
       </c>
       <c r="C25" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D25" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>9</v>
+        <v>Equipment</v>
+      </c>
+      <c r="E25" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F25" s="1">
-        <v>26</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>44</v>
       </c>
       <c r="G25" s="1"/>
     </row>
@@ -1220,21 +1259,23 @@
       </c>
       <c r="B26" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46115</v>
+        <v>46149</v>
       </c>
       <c r="C26" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D26" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>9</v>
+        <v>Perssonel</v>
+      </c>
+      <c r="E26" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F26" s="1">
-        <v>28</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>13</v>
       </c>
       <c r="G26" s="1"/>
     </row>
@@ -1245,21 +1286,23 @@
       </c>
       <c r="B27" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46164</v>
+        <v>46145</v>
       </c>
       <c r="C27" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D27" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>Perssonel</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>9</v>
+      <c r="E27" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F27" s="1">
-        <v>29</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>25</v>
       </c>
       <c r="G27" s="1"/>
     </row>
@@ -1270,21 +1313,23 @@
       </c>
       <c r="B28" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46149</v>
+        <v>46154</v>
       </c>
       <c r="C28" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Packaging</v>
       </c>
       <c r="D28" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>Perssonel</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>8</v>
+      <c r="E28" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Reject</v>
       </c>
       <c r="F28" s="1">
-        <v>31</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>29</v>
       </c>
       <c r="G28" s="1"/>
     </row>
@@ -1295,7 +1340,7 @@
       </c>
       <c r="B29" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46128</v>
+        <v>46133</v>
       </c>
       <c r="C29" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1303,13 +1348,15 @@
       </c>
       <c r="D29" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>8</v>
+        <v>Materials</v>
+      </c>
+      <c r="E29" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F29" s="1">
-        <v>13</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>24</v>
       </c>
       <c r="G29" s="1"/>
     </row>
@@ -1320,21 +1367,23 @@
       </c>
       <c r="B30" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46166</v>
+        <v>46115</v>
       </c>
       <c r="C30" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D30" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>8</v>
+        <v>Supplies</v>
+      </c>
+      <c r="E30" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F30" s="1">
-        <v>12</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>24</v>
       </c>
       <c r="G30" s="1"/>
     </row>
@@ -1345,21 +1394,23 @@
       </c>
       <c r="B31" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46161</v>
+        <v>46160</v>
       </c>
       <c r="C31" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Field opetations</v>
       </c>
       <c r="D31" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
         <v>Supplies</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>8</v>
+      <c r="E31" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F31" s="1">
-        <v>10</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>45</v>
       </c>
       <c r="G31" s="1"/>
     </row>
@@ -1370,26 +1421,27 @@
       </c>
       <c r="B32" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46118</v>
+        <v>46115</v>
       </c>
       <c r="C32" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Field opetations</v>
       </c>
       <c r="D32" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>8</v>
+        <v>Materials</v>
+      </c>
+      <c r="E32" s="1" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v>Approved</v>
       </c>
       <c r="F32" s="1">
-        <v>27</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>17</v>
       </c>
       <c r="G32" s="1"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="9"/>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D33" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
We complete the rejection reason field using an Excel formula
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E40C24-8FA5-4A73-874C-907A54DD6A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A30E4F0-A199-4216-95A6-E01FBBF746B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -63,18 +63,6 @@
   </si>
   <si>
     <t>Rejection reason</t>
-  </si>
-  <si>
-    <t>Bugget Exceeded</t>
-  </si>
-  <si>
-    <t>Imcomplete information</t>
-  </si>
-  <si>
-    <t>Not justified</t>
-  </si>
-  <si>
-    <t>Duplicate Request</t>
   </si>
 </sst>
 </file>
@@ -183,18 +171,97 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -585,15 +652,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.2" x14ac:dyDescent="0.5">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -628,25 +695,28 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46155</v>
+        <v>46128</v>
       </c>
       <c r="C3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
-        <v>Logistics</v>
+        <v>Field opetations</v>
       </c>
       <c r="D3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
-        <v>Materials</v>
+        <v>Supplies</v>
       </c>
       <c r="E3" s="1" t="str">
-        <f ca="1">IF(RAND()&lt;0.7,"Approved","Reject")</f>
-        <v>Reject</v>
+        <f ca="1">IF(RAND()&lt;0.7,"Approved","Rejected")</f>
+        <v>Approved</v>
       </c>
       <c r="F3" s="1">
         <f ca="1">RANDBETWEEN(4,48)</f>
-        <v>20</v>
-      </c>
-      <c r="G3" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="G3" s="1" t="str">
+        <f ca="1">IF(E3="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="str">
@@ -655,7 +725,7 @@
       </c>
       <c r="B4" s="4">
         <f t="shared" ref="B4:B32" ca="1" si="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46162</v>
+        <v>46166</v>
       </c>
       <c r="C4" s="1" t="str">
         <f t="shared" ref="C4:C32" ca="1" si="2">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
@@ -666,14 +736,17 @@
         <v>Equipment</v>
       </c>
       <c r="E4" s="1" t="str">
-        <f t="shared" ref="E4:E32" ca="1" si="4">IF(RAND()&lt;0.7,"Approved","Reject")</f>
+        <f t="shared" ref="E4:E32" ca="1" si="4">IF(RAND()&lt;0.7,"Approved","Rejected")</f>
         <v>Approved</v>
       </c>
       <c r="F4" s="1">
         <f t="shared" ref="F4:F32" ca="1" si="5">RANDBETWEEN(4,48)</f>
-        <v>32</v>
-      </c>
-      <c r="G4" s="1"/>
+        <v>26</v>
+      </c>
+      <c r="G4" s="1" t="str">
+        <f t="shared" ref="G4:G33" ca="1" si="6">IF(E4="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="str">
@@ -682,11 +755,11 @@
       </c>
       <c r="B5" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46122</v>
+        <v>46115</v>
       </c>
       <c r="C5" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D5" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -694,13 +767,16 @@
       </c>
       <c r="E5" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Approved</v>
       </c>
       <c r="F5" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>23</v>
-      </c>
-      <c r="G5" s="1"/>
+        <v>12</v>
+      </c>
+      <c r="G5" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="str">
@@ -709,25 +785,28 @@
       </c>
       <c r="B6" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46143</v>
+        <v>46163</v>
       </c>
       <c r="C6" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Administration</v>
       </c>
       <c r="D6" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Materials</v>
       </c>
       <c r="E6" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F6" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>41</v>
-      </c>
-      <c r="G6" s="1"/>
+        <v>29</v>
+      </c>
+      <c r="G6" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Duplicate request</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="str">
@@ -736,11 +815,11 @@
       </c>
       <c r="B7" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46130</v>
+        <v>46124</v>
       </c>
       <c r="C7" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Field opetations</v>
       </c>
       <c r="D7" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -748,13 +827,16 @@
       </c>
       <c r="E7" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Approved</v>
       </c>
       <c r="F7" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="G7" s="1"/>
+        <v>6</v>
+      </c>
+      <c r="G7" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="str">
@@ -763,15 +845,15 @@
       </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46124</v>
+        <v>46151</v>
       </c>
       <c r="C8" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D8" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Perssonel</v>
       </c>
       <c r="E8" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -779,10 +861,11 @@
       </c>
       <c r="F8" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>10</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>8</v>
+        <v>26</v>
+      </c>
+      <c r="G8" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -792,15 +875,15 @@
       </c>
       <c r="B9" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46121</v>
+        <v>46165</v>
       </c>
       <c r="C9" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D9" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Equipment</v>
       </c>
       <c r="E9" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -808,10 +891,11 @@
       </c>
       <c r="F9" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>25</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
+      </c>
+      <c r="G9" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -821,15 +905,15 @@
       </c>
       <c r="B10" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46128</v>
+        <v>46122</v>
       </c>
       <c r="C10" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Administration</v>
       </c>
       <c r="D10" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Equipment</v>
       </c>
       <c r="E10" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -837,10 +921,11 @@
       </c>
       <c r="F10" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>26</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>10</v>
+        <v>38</v>
+      </c>
+      <c r="G10" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -850,7 +935,7 @@
       </c>
       <c r="B11" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46157</v>
+        <v>46125</v>
       </c>
       <c r="C11" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -858,7 +943,7 @@
       </c>
       <c r="D11" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Materials</v>
       </c>
       <c r="E11" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -866,9 +951,12 @@
       </c>
       <c r="F11" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>44</v>
-      </c>
-      <c r="G11" s="1"/>
+        <v>9</v>
+      </c>
+      <c r="G11" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="str">
@@ -877,26 +965,27 @@
       </c>
       <c r="B12" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46145</v>
+        <v>46129</v>
       </c>
       <c r="C12" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Field opetations</v>
       </c>
       <c r="D12" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Supplies</v>
       </c>
       <c r="E12" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F12" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>16</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
+      </c>
+      <c r="G12" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Duplicate request</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -906,15 +995,15 @@
       </c>
       <c r="B13" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46161</v>
+        <v>46116</v>
       </c>
       <c r="C13" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Field opetations</v>
       </c>
       <c r="D13" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Equipment</v>
       </c>
       <c r="E13" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -922,10 +1011,11 @@
       </c>
       <c r="F13" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>24</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
+      </c>
+      <c r="G13" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -935,15 +1025,15 @@
       </c>
       <c r="B14" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46162</v>
+        <v>46149</v>
       </c>
       <c r="C14" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D14" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Perssonel</v>
       </c>
       <c r="E14" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -951,9 +1041,12 @@
       </c>
       <c r="F14" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>39</v>
-      </c>
-      <c r="G14" s="6"/>
+        <v>38</v>
+      </c>
+      <c r="G14" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="str">
@@ -962,15 +1055,15 @@
       </c>
       <c r="B15" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46158</v>
+        <v>46143</v>
       </c>
       <c r="C15" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D15" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Materials</v>
       </c>
       <c r="E15" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -978,9 +1071,12 @@
       </c>
       <c r="F15" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>9</v>
-      </c>
-      <c r="G15" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="G15" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="str">
@@ -989,25 +1085,28 @@
       </c>
       <c r="B16" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46146</v>
+        <v>46125</v>
       </c>
       <c r="C16" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D16" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Supplies</v>
       </c>
       <c r="E16" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Rejected</v>
       </c>
       <c r="F16" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>47</v>
-      </c>
-      <c r="G16" s="1"/>
+        <v>41</v>
+      </c>
+      <c r="G16" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Imcomplete information</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="str">
@@ -1016,7 +1115,7 @@
       </c>
       <c r="B17" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46140</v>
+        <v>46152</v>
       </c>
       <c r="C17" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1024,7 +1123,7 @@
       </c>
       <c r="D17" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Materials</v>
       </c>
       <c r="E17" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1032,9 +1131,12 @@
       </c>
       <c r="F17" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>9</v>
-      </c>
-      <c r="G17" s="1"/>
+        <v>39</v>
+      </c>
+      <c r="G17" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="str">
@@ -1043,11 +1145,11 @@
       </c>
       <c r="B18" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46147</v>
+        <v>46149</v>
       </c>
       <c r="C18" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Logistics</v>
       </c>
       <c r="D18" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1055,13 +1157,16 @@
       </c>
       <c r="E18" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Approved</v>
       </c>
       <c r="F18" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="G18" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="G18" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="str">
@@ -1070,7 +1175,7 @@
       </c>
       <c r="B19" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46126</v>
+        <v>46166</v>
       </c>
       <c r="C19" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1078,7 +1183,7 @@
       </c>
       <c r="D19" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Supplies</v>
       </c>
       <c r="E19" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1086,9 +1191,12 @@
       </c>
       <c r="F19" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>44</v>
-      </c>
-      <c r="G19" s="1"/>
+        <v>8</v>
+      </c>
+      <c r="G19" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="str">
@@ -1097,7 +1205,7 @@
       </c>
       <c r="B20" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46118</v>
+        <v>46163</v>
       </c>
       <c r="C20" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1105,17 +1213,20 @@
       </c>
       <c r="D20" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Equipment</v>
       </c>
       <c r="E20" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Approved</v>
       </c>
       <c r="F20" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>28</v>
-      </c>
-      <c r="G20" s="1"/>
+        <v>26</v>
+      </c>
+      <c r="G20" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="str">
@@ -1124,25 +1235,28 @@
       </c>
       <c r="B21" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46124</v>
+        <v>46142</v>
       </c>
       <c r="C21" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D21" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Materials</v>
       </c>
       <c r="E21" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Approved</v>
       </c>
       <c r="F21" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>29</v>
-      </c>
-      <c r="G21" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="G21" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="str">
@@ -1151,7 +1265,7 @@
       </c>
       <c r="B22" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46160</v>
+        <v>46139</v>
       </c>
       <c r="C22" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1159,7 +1273,7 @@
       </c>
       <c r="D22" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Materials</v>
       </c>
       <c r="E22" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1167,9 +1281,12 @@
       </c>
       <c r="F22" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>17</v>
-      </c>
-      <c r="G22" s="1"/>
+        <v>41</v>
+      </c>
+      <c r="G22" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="str">
@@ -1178,25 +1295,28 @@
       </c>
       <c r="B23" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46141</v>
+        <v>46145</v>
       </c>
       <c r="C23" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Field opetations</v>
       </c>
       <c r="D23" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Supplies</v>
       </c>
       <c r="E23" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Approved</v>
       </c>
       <c r="F23" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>35</v>
-      </c>
-      <c r="G23" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="G23" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="str">
@@ -1205,11 +1325,11 @@
       </c>
       <c r="B24" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46124</v>
+        <v>46153</v>
       </c>
       <c r="C24" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D24" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1217,13 +1337,16 @@
       </c>
       <c r="E24" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F24" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>32</v>
-      </c>
-      <c r="G24" s="1"/>
+        <v>6</v>
+      </c>
+      <c r="G24" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Imcomplete information</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="str">
@@ -1232,7 +1355,7 @@
       </c>
       <c r="B25" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46145</v>
+        <v>46144</v>
       </c>
       <c r="C25" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1244,13 +1367,16 @@
       </c>
       <c r="E25" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F25" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>44</v>
-      </c>
-      <c r="G25" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="G25" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Imcomplete information</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="str">
@@ -1259,15 +1385,15 @@
       </c>
       <c r="B26" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="C26" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D26" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Equipment</v>
       </c>
       <c r="E26" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1275,9 +1401,12 @@
       </c>
       <c r="F26" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>13</v>
-      </c>
-      <c r="G26" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="G26" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="str">
@@ -1286,25 +1415,28 @@
       </c>
       <c r="B27" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46145</v>
+        <v>46144</v>
       </c>
       <c r="C27" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Logistics</v>
       </c>
       <c r="D27" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Materials</v>
       </c>
       <c r="E27" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F27" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>25</v>
-      </c>
-      <c r="G27" s="1"/>
+        <v>8</v>
+      </c>
+      <c r="G27" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Imcomplete information</v>
+      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="str">
@@ -1313,7 +1445,7 @@
       </c>
       <c r="B28" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46154</v>
+        <v>46116</v>
       </c>
       <c r="C28" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1321,17 +1453,20 @@
       </c>
       <c r="D28" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Materials</v>
       </c>
       <c r="E28" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Reject</v>
+        <v>Rejected</v>
       </c>
       <c r="F28" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>29</v>
-      </c>
-      <c r="G28" s="1"/>
+        <v>9</v>
+      </c>
+      <c r="G28" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Imcomplete information</v>
+      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="str">
@@ -1340,11 +1475,11 @@
       </c>
       <c r="B29" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46133</v>
+        <v>46140</v>
       </c>
       <c r="C29" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D29" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1356,9 +1491,12 @@
       </c>
       <c r="F29" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>24</v>
-      </c>
-      <c r="G29" s="1"/>
+        <v>37</v>
+      </c>
+      <c r="G29" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="str">
@@ -1367,11 +1505,11 @@
       </c>
       <c r="B30" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="C30" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D30" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1383,9 +1521,12 @@
       </c>
       <c r="F30" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>24</v>
-      </c>
-      <c r="G30" s="1"/>
+        <v>40</v>
+      </c>
+      <c r="G30" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="str">
@@ -1394,25 +1535,28 @@
       </c>
       <c r="B31" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46160</v>
+        <v>46168</v>
       </c>
       <c r="C31" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Administration</v>
       </c>
       <c r="D31" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Equipment</v>
       </c>
       <c r="E31" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F31" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>45</v>
-      </c>
-      <c r="G31" s="1"/>
+        <v>30</v>
+      </c>
+      <c r="G31" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Bugget</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="str">
@@ -1421,15 +1565,15 @@
       </c>
       <c r="B32" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46115</v>
+        <v>46139</v>
       </c>
       <c r="C32" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Administration</v>
       </c>
       <c r="D32" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Perssonel</v>
       </c>
       <c r="E32" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1437,18 +1581,30 @@
       </c>
       <c r="F32" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>17</v>
-      </c>
-      <c r="G32" s="1"/>
-    </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G32" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D33" s="5"/>
+      <c r="G33" s="8" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="E1:E1048576">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Rejected">
+      <formula>NOT(ISERROR(SEARCH("Rejected",E1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
add conditional format in field rejection reason
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A30E4F0-A199-4216-95A6-E01FBBF746B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54AE7BCC-4A17-45D7-9BE2-555EAA5B30E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -164,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -177,12 +177,31 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -695,15 +714,15 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46128</v>
+        <v>46170</v>
       </c>
       <c r="C3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
-        <v>Supplies</v>
+        <v>Perssonel</v>
       </c>
       <c r="E3" s="1" t="str">
         <f ca="1">IF(RAND()&lt;0.7,"Approved","Rejected")</f>
@@ -711,11 +730,11 @@
       </c>
       <c r="F3" s="1">
         <f ca="1">RANDBETWEEN(4,48)</f>
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G3" s="1" t="str">
-        <f ca="1">IF(E3="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"")</f>
-        <v/>
+        <f ca="1">IF(E3="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"Not necesary")</f>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -725,27 +744,27 @@
       </c>
       <c r="B4" s="4">
         <f t="shared" ref="B4:B32" ca="1" si="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46166</v>
+        <v>46122</v>
       </c>
       <c r="C4" s="1" t="str">
         <f t="shared" ref="C4:C32" ca="1" si="2">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D4" s="1" t="str">
         <f t="shared" ref="D4:D32" ca="1" si="3">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
-        <v>Equipment</v>
+        <v>Materials</v>
       </c>
       <c r="E4" s="1" t="str">
         <f t="shared" ref="E4:E32" ca="1" si="4">IF(RAND()&lt;0.7,"Approved","Rejected")</f>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F4" s="1">
         <f t="shared" ref="F4:F32" ca="1" si="5">RANDBETWEEN(4,48)</f>
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G4" s="1" t="str">
-        <f t="shared" ref="G4:G33" ca="1" si="6">IF(E4="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"")</f>
-        <v/>
+        <f t="shared" ref="G4:G33" ca="1" si="6">IF(E4="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"Not necesary")</f>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -755,7 +774,7 @@
       </c>
       <c r="B5" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46115</v>
+        <v>46165</v>
       </c>
       <c r="C5" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -763,7 +782,7 @@
       </c>
       <c r="D5" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Supplies</v>
       </c>
       <c r="E5" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -771,11 +790,11 @@
       </c>
       <c r="F5" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G5" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -785,27 +804,27 @@
       </c>
       <c r="B6" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46163</v>
+        <v>46139</v>
       </c>
       <c r="C6" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Field opetations</v>
       </c>
       <c r="D6" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Equipment</v>
       </c>
       <c r="E6" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F6" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="G6" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Duplicate request</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -815,15 +834,15 @@
       </c>
       <c r="B7" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46124</v>
+        <v>46164</v>
       </c>
       <c r="C7" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Administration</v>
       </c>
       <c r="D7" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Perssonel</v>
       </c>
       <c r="E7" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -831,11 +850,11 @@
       </c>
       <c r="F7" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="G7" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -845,27 +864,27 @@
       </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46151</v>
+        <v>46140</v>
       </c>
       <c r="C8" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Field opetations</v>
       </c>
       <c r="D8" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Materials</v>
       </c>
       <c r="E8" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F8" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G8" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not justifed</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -875,15 +894,15 @@
       </c>
       <c r="B9" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46165</v>
+        <v>46154</v>
       </c>
       <c r="C9" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Field opetations</v>
       </c>
       <c r="D9" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Materials</v>
       </c>
       <c r="E9" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -891,11 +910,11 @@
       </c>
       <c r="F9" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G9" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -905,11 +924,11 @@
       </c>
       <c r="B10" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46122</v>
+        <v>46169</v>
       </c>
       <c r="C10" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Logistics</v>
       </c>
       <c r="D10" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -921,11 +940,11 @@
       </c>
       <c r="F10" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="G10" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -935,11 +954,11 @@
       </c>
       <c r="B11" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46125</v>
+        <v>46144</v>
       </c>
       <c r="C11" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D11" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -951,11 +970,11 @@
       </c>
       <c r="F11" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="G11" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -965,7 +984,7 @@
       </c>
       <c r="B12" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46129</v>
+        <v>46117</v>
       </c>
       <c r="C12" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -981,11 +1000,11 @@
       </c>
       <c r="F12" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="G12" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Duplicate request</v>
+        <v>Imcomplete information</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -995,7 +1014,7 @@
       </c>
       <c r="B13" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46116</v>
+        <v>46125</v>
       </c>
       <c r="C13" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1003,7 +1022,7 @@
       </c>
       <c r="D13" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Materials</v>
       </c>
       <c r="E13" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1011,11 +1030,11 @@
       </c>
       <c r="F13" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="G13" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -1025,27 +1044,27 @@
       </c>
       <c r="B14" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46149</v>
+        <v>46152</v>
       </c>
       <c r="C14" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Packaging</v>
       </c>
       <c r="D14" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Supplies</v>
       </c>
       <c r="E14" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F14" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="G14" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1055,27 +1074,27 @@
       </c>
       <c r="B15" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46143</v>
+        <v>46139</v>
       </c>
       <c r="C15" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D15" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Supplies</v>
       </c>
       <c r="E15" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F15" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G15" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Imcomplete information</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -1085,11 +1104,11 @@
       </c>
       <c r="B16" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46125</v>
+        <v>46140</v>
       </c>
       <c r="C16" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D16" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1097,15 +1116,15 @@
       </c>
       <c r="E16" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F16" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="G16" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Imcomplete information</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -1115,15 +1134,15 @@
       </c>
       <c r="B17" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46152</v>
+        <v>46160</v>
       </c>
       <c r="C17" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Field opetations</v>
       </c>
       <c r="D17" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Equipment</v>
       </c>
       <c r="E17" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1131,11 +1150,11 @@
       </c>
       <c r="F17" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="G17" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1145,11 +1164,11 @@
       </c>
       <c r="B18" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46149</v>
+        <v>46124</v>
       </c>
       <c r="C18" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D18" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1157,15 +1176,15 @@
       </c>
       <c r="E18" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F18" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G18" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1175,7 +1194,7 @@
       </c>
       <c r="B19" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46166</v>
+        <v>46131</v>
       </c>
       <c r="C19" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1183,19 +1202,19 @@
       </c>
       <c r="D19" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Equipment</v>
       </c>
       <c r="E19" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F19" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="G19" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1205,7 +1224,7 @@
       </c>
       <c r="B20" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46163</v>
+        <v>46157</v>
       </c>
       <c r="C20" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1213,7 +1232,7 @@
       </c>
       <c r="D20" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Perssonel</v>
       </c>
       <c r="E20" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1221,11 +1240,11 @@
       </c>
       <c r="F20" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G20" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -1235,7 +1254,7 @@
       </c>
       <c r="B21" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46142</v>
+        <v>46126</v>
       </c>
       <c r="C21" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1247,15 +1266,15 @@
       </c>
       <c r="E21" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F21" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G21" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not justifed</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1265,11 +1284,11 @@
       </c>
       <c r="B22" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46114</v>
       </c>
       <c r="C22" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D22" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1281,11 +1300,11 @@
       </c>
       <c r="F22" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="G22" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -1295,7 +1314,7 @@
       </c>
       <c r="B23" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46145</v>
+        <v>46119</v>
       </c>
       <c r="C23" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1303,7 +1322,7 @@
       </c>
       <c r="D23" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Perssonel</v>
       </c>
       <c r="E23" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1311,11 +1330,11 @@
       </c>
       <c r="F23" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="G23" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -1325,11 +1344,11 @@
       </c>
       <c r="B24" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46153</v>
+        <v>46159</v>
       </c>
       <c r="C24" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Field opetations</v>
       </c>
       <c r="D24" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1337,15 +1356,15 @@
       </c>
       <c r="E24" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F24" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="G24" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Imcomplete information</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1355,15 +1374,15 @@
       </c>
       <c r="B25" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46144</v>
+        <v>46135</v>
       </c>
       <c r="C25" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D25" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Perssonel</v>
       </c>
       <c r="E25" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1371,11 +1390,11 @@
       </c>
       <c r="F25" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="G25" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Imcomplete information</v>
+        <v>Duplicate request</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1385,15 +1404,15 @@
       </c>
       <c r="B26" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46153</v>
+        <v>46166</v>
       </c>
       <c r="C26" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D26" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Supplies</v>
       </c>
       <c r="E26" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1401,11 +1420,11 @@
       </c>
       <c r="F26" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="G26" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1415,27 +1434,27 @@
       </c>
       <c r="B27" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46144</v>
+        <v>46134</v>
       </c>
       <c r="C27" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Administration</v>
       </c>
       <c r="D27" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Perssonel</v>
       </c>
       <c r="E27" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F27" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G27" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Imcomplete information</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1445,15 +1464,15 @@
       </c>
       <c r="B28" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46116</v>
+        <v>46157</v>
       </c>
       <c r="C28" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D28" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Supplies</v>
       </c>
       <c r="E28" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1461,11 +1480,11 @@
       </c>
       <c r="F28" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="G28" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Imcomplete information</v>
+        <v>Not justifed</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1475,15 +1494,15 @@
       </c>
       <c r="B29" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46140</v>
+        <v>46118</v>
       </c>
       <c r="C29" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D29" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Equipment</v>
       </c>
       <c r="E29" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1491,11 +1510,11 @@
       </c>
       <c r="F29" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="G29" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
@@ -1505,7 +1524,7 @@
       </c>
       <c r="B30" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46126</v>
+        <v>46159</v>
       </c>
       <c r="C30" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1513,7 +1532,7 @@
       </c>
       <c r="D30" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Materials</v>
       </c>
       <c r="E30" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1521,11 +1540,11 @@
       </c>
       <c r="F30" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="G30" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
@@ -1535,15 +1554,15 @@
       </c>
       <c r="B31" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46168</v>
+        <v>46167</v>
       </c>
       <c r="C31" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D31" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Materials</v>
       </c>
       <c r="E31" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1551,7 +1570,7 @@
       </c>
       <c r="F31" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G31" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1565,15 +1584,15 @@
       </c>
       <c r="B32" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46150</v>
       </c>
       <c r="C32" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D32" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Perssonel</v>
+        <v>Supplies</v>
       </c>
       <c r="E32" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1581,18 +1600,18 @@
       </c>
       <c r="F32" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="G32" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D33" s="5"/>
-      <c r="G33" s="8" t="str">
-        <f t="shared" ca="1" si="6"/>
-        <v/>
+      <c r="G33" s="1" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Not necesary</v>
       </c>
     </row>
   </sheetData>
@@ -1601,8 +1620,13 @@
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Rejected">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Rejected">
       <formula>NOT(ISERROR(SEARCH("Rejected",E1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1:G1048576">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Not necesary">
+      <formula>NOT(ISERROR(SEARCH("Not necesary",G1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add new sheet with a excfel formula
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54AE7BCC-4A17-45D7-9BE2-555EAA5B30E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54943612-D0D0-4B1C-8571-FE733D7FBEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA" sheetId="1" r:id="rId1"/>
+    <sheet name="Excel Formula" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -63,6 +64,39 @@
   </si>
   <si>
     <t>Rejection reason</t>
+  </si>
+  <si>
+    <t>Request Type</t>
+  </si>
+  <si>
+    <t>Response Time(Hrs)</t>
+  </si>
+  <si>
+    <t>Rejection Reason</t>
+  </si>
+  <si>
+    <t>Excel Formulas</t>
+  </si>
+  <si>
+    <t>=REQ-"&amp;TEXT(ROW()-2;"000")</t>
+  </si>
+  <si>
+    <t>=Date(2026;04;01)+int(RAND()*59)</t>
+  </si>
+  <si>
+    <t>=CHOOSE(RANDBETWEEN(1;4);"Materials";"Personnel";"Equipment";"Supplies")</t>
+  </si>
+  <si>
+    <t>=CHOOSE(RANDBETWEEN(1;4);"FieldOperations";"Packaging";"Administration";"Logistic")</t>
+  </si>
+  <si>
+    <t>=if(RAND()&lt;0,7;"Approved";"Rejected")</t>
+  </si>
+  <si>
+    <t>=RANDBETWEEN(1;48)</t>
+  </si>
+  <si>
+    <t>=IF(F3="Rejected";CHOOSE(RANDBETWEEN(1;4);"Budget";"Incomplete information";"Not justified";"Duplicate request")</t>
   </si>
 </sst>
 </file>
@@ -113,7 +147,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -160,11 +194,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -177,11 +224,35 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -714,7 +785,7 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46170</v>
+        <v>46119</v>
       </c>
       <c r="C3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
@@ -722,19 +793,19 @@
       </c>
       <c r="D3" s="1" t="str">
         <f ca="1">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
-        <v>Perssonel</v>
+        <v>Equipment</v>
       </c>
       <c r="E3" s="1" t="str">
         <f ca="1">IF(RAND()&lt;0.7,"Approved","Rejected")</f>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F3" s="1">
         <f ca="1">RANDBETWEEN(4,48)</f>
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G3" s="1" t="str">
         <f ca="1">IF(E3="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"Not necesary")</f>
-        <v>Not necesary</v>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -744,27 +815,27 @@
       </c>
       <c r="B4" s="4">
         <f t="shared" ref="B4:B32" ca="1" si="1">DATE(2026,4,1)+INT(RAND()*59)</f>
-        <v>46122</v>
+        <v>46153</v>
       </c>
       <c r="C4" s="1" t="str">
         <f t="shared" ref="C4:C32" ca="1" si="2">CHOOSE(RANDBETWEEN(1,4),"Field opetations","Packaging","Administration","Logistics")</f>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D4" s="1" t="str">
         <f t="shared" ref="D4:D32" ca="1" si="3">CHOOSE(RANDBETWEEN(1,4),"Materials","Perssonel","Equipment","Supplies")</f>
-        <v>Materials</v>
+        <v>Supplies</v>
       </c>
       <c r="E4" s="1" t="str">
         <f t="shared" ref="E4:E32" ca="1" si="4">IF(RAND()&lt;0.7,"Approved","Rejected")</f>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F4" s="1">
         <f t="shared" ref="F4:F32" ca="1" si="5">RANDBETWEEN(4,48)</f>
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="G4" s="1" t="str">
         <f t="shared" ref="G4:G33" ca="1" si="6">IF(E4="Rejected",CHOOSE(RANDBETWEEN(1,4),"Bugget","Imcomplete information","Not justifed","Duplicate request"),"Not necesary")</f>
-        <v>Bugget</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -774,15 +845,15 @@
       </c>
       <c r="B5" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46165</v>
+        <v>46145</v>
       </c>
       <c r="C5" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Packaging</v>
       </c>
       <c r="D5" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Equipment</v>
       </c>
       <c r="E5" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -790,7 +861,7 @@
       </c>
       <c r="F5" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G5" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -804,15 +875,15 @@
       </c>
       <c r="B6" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46158</v>
       </c>
       <c r="C6" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D6" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Perssonel</v>
       </c>
       <c r="E6" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -820,7 +891,7 @@
       </c>
       <c r="F6" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="G6" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -834,7 +905,7 @@
       </c>
       <c r="B7" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46164</v>
+        <v>46152</v>
       </c>
       <c r="C7" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -846,15 +917,15 @@
       </c>
       <c r="E7" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F7" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="G7" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not necesary</v>
+        <v>Not justifed</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -864,7 +935,7 @@
       </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46140</v>
+        <v>46115</v>
       </c>
       <c r="C8" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -876,15 +947,15 @@
       </c>
       <c r="E8" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F8" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="G8" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not justifed</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -894,15 +965,15 @@
       </c>
       <c r="B9" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46154</v>
+        <v>46158</v>
       </c>
       <c r="C9" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D9" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Perssonel</v>
       </c>
       <c r="E9" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -910,7 +981,7 @@
       </c>
       <c r="F9" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G9" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -924,27 +995,27 @@
       </c>
       <c r="B10" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46169</v>
+        <v>46129</v>
       </c>
       <c r="C10" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Field opetations</v>
       </c>
       <c r="D10" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Supplies</v>
       </c>
       <c r="E10" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F10" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G10" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not necesary</v>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -954,7 +1025,7 @@
       </c>
       <c r="B11" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46144</v>
+        <v>46121</v>
       </c>
       <c r="C11" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -962,7 +1033,7 @@
       </c>
       <c r="D11" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Perssonel</v>
       </c>
       <c r="E11" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -970,7 +1041,7 @@
       </c>
       <c r="F11" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G11" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -984,27 +1055,27 @@
       </c>
       <c r="B12" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46117</v>
+        <v>46166</v>
       </c>
       <c r="C12" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D12" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Perssonel</v>
       </c>
       <c r="E12" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F12" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="G12" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Imcomplete information</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -1014,27 +1085,27 @@
       </c>
       <c r="B13" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46125</v>
+        <v>46164</v>
       </c>
       <c r="C13" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Field opetations</v>
+        <v>Logistics</v>
       </c>
       <c r="D13" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Equipment</v>
       </c>
       <c r="E13" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F13" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="G13" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not necesary</v>
+        <v>Duplicate request</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -1044,15 +1115,15 @@
       </c>
       <c r="B14" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46152</v>
+        <v>46131</v>
       </c>
       <c r="C14" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D14" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Perssonel</v>
       </c>
       <c r="E14" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1060,11 +1131,11 @@
       </c>
       <c r="F14" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="G14" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Bugget</v>
+        <v>Imcomplete information</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1074,7 +1145,7 @@
       </c>
       <c r="B15" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46146</v>
       </c>
       <c r="C15" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1082,7 +1153,7 @@
       </c>
       <c r="D15" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Equipment</v>
       </c>
       <c r="E15" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1090,11 +1161,11 @@
       </c>
       <c r="F15" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G15" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Imcomplete information</v>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -1104,11 +1175,11 @@
       </c>
       <c r="B16" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46140</v>
+        <v>46146</v>
       </c>
       <c r="C16" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D16" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1120,7 +1191,7 @@
       </c>
       <c r="F16" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="G16" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1134,7 +1205,7 @@
       </c>
       <c r="B17" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46160</v>
+        <v>46117</v>
       </c>
       <c r="C17" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1142,7 +1213,7 @@
       </c>
       <c r="D17" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Supplies</v>
       </c>
       <c r="E17" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1164,27 +1235,27 @@
       </c>
       <c r="B18" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46124</v>
+        <v>46113</v>
       </c>
       <c r="C18" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Packaging</v>
       </c>
       <c r="D18" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Materials</v>
       </c>
       <c r="E18" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F18" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="G18" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Bugget</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1194,15 +1265,15 @@
       </c>
       <c r="B19" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46131</v>
+        <v>46152</v>
       </c>
       <c r="C19" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D19" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Perssonel</v>
       </c>
       <c r="E19" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1210,11 +1281,11 @@
       </c>
       <c r="F19" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G19" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Bugget</v>
+        <v>Imcomplete information</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1224,11 +1295,11 @@
       </c>
       <c r="B20" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46157</v>
+        <v>46128</v>
       </c>
       <c r="C20" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Packaging</v>
       </c>
       <c r="D20" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1240,7 +1311,7 @@
       </c>
       <c r="F20" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="G20" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1254,27 +1325,27 @@
       </c>
       <c r="B21" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46126</v>
+        <v>46169</v>
       </c>
       <c r="C21" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Logistics</v>
       </c>
       <c r="D21" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Perssonel</v>
       </c>
       <c r="E21" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F21" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G21" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not justifed</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1284,15 +1355,15 @@
       </c>
       <c r="B22" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46114</v>
+        <v>46148</v>
       </c>
       <c r="C22" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Field opetations</v>
       </c>
       <c r="D22" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Perssonel</v>
       </c>
       <c r="E22" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1300,7 +1371,7 @@
       </c>
       <c r="F22" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="G22" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1314,7 +1385,7 @@
       </c>
       <c r="B23" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46119</v>
+        <v>46171</v>
       </c>
       <c r="C23" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1326,15 +1397,15 @@
       </c>
       <c r="E23" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F23" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G23" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not necesary</v>
+        <v>Imcomplete information</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -1344,7 +1415,7 @@
       </c>
       <c r="B24" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46159</v>
+        <v>46145</v>
       </c>
       <c r="C24" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -1352,19 +1423,19 @@
       </c>
       <c r="D24" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Perssonel</v>
       </c>
       <c r="E24" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Approved</v>
+        <v>Rejected</v>
       </c>
       <c r="F24" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="G24" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not necesary</v>
+        <v>Bugget</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1374,11 +1445,11 @@
       </c>
       <c r="B25" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46135</v>
+        <v>46138</v>
       </c>
       <c r="C25" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Field opetations</v>
       </c>
       <c r="D25" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1390,7 +1461,7 @@
       </c>
       <c r="F25" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="G25" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1404,15 +1475,15 @@
       </c>
       <c r="B26" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46166</v>
+        <v>46171</v>
       </c>
       <c r="C26" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D26" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Materials</v>
       </c>
       <c r="E26" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1420,7 +1491,7 @@
       </c>
       <c r="F26" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G26" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1434,11 +1505,11 @@
       </c>
       <c r="B27" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46134</v>
+        <v>46140</v>
       </c>
       <c r="C27" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Administration</v>
+        <v>Field opetations</v>
       </c>
       <c r="D27" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1450,7 +1521,7 @@
       </c>
       <c r="F27" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G27" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1464,27 +1535,27 @@
       </c>
       <c r="B28" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46157</v>
+        <v>46167</v>
       </c>
       <c r="C28" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Logistics</v>
+        <v>Field opetations</v>
       </c>
       <c r="D28" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Equipment</v>
       </c>
       <c r="E28" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F28" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="G28" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
-        <v>Not justifed</v>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1494,15 +1565,15 @@
       </c>
       <c r="B29" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46118</v>
+        <v>46148</v>
       </c>
       <c r="C29" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D29" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Equipment</v>
+        <v>Perssonel</v>
       </c>
       <c r="E29" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1510,7 +1581,7 @@
       </c>
       <c r="F29" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G29" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1532,7 +1603,7 @@
       </c>
       <c r="D30" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Materials</v>
+        <v>Supplies</v>
       </c>
       <c r="E30" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -1540,7 +1611,7 @@
       </c>
       <c r="F30" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G30" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1558,7 +1629,7 @@
       </c>
       <c r="C31" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Administration</v>
       </c>
       <c r="D31" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -1566,15 +1637,15 @@
       </c>
       <c r="E31" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>Rejected</v>
+        <v>Approved</v>
       </c>
       <c r="F31" s="1">
         <f t="shared" ca="1" si="5"/>
-        <v>10</v>
-      </c>
-      <c r="G31" s="1" t="str">
-        <f t="shared" ca="1" si="6"/>
-        <v>Bugget</v>
+        <v>12</v>
+      </c>
+      <c r="G31" s="8" t="str">
+        <f t="shared" ca="1" si="6"/>
+        <v>Not necesary</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
@@ -1584,23 +1655,23 @@
       </c>
       <c r="B32" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>46150</v>
+        <v>46115</v>
       </c>
       <c r="C32" s="1" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>Packaging</v>
+        <v>Logistics</v>
       </c>
       <c r="D32" s="1" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Supplies</v>
+        <v>Materials</v>
       </c>
       <c r="E32" s="1" t="str">
         <f t="shared" ca="1" si="4"/>
         <v>Approved</v>
       </c>
-      <c r="F32" s="1">
-        <f t="shared" ca="1" si="5"/>
-        <v>42</v>
+      <c r="F32" s="10">
+        <f t="shared" ca="1" si="5"/>
+        <v>6</v>
       </c>
       <c r="G32" s="1" t="str">
         <f t="shared" ca="1" si="6"/>
@@ -1609,10 +1680,7 @@
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D33" s="5"/>
-      <c r="G33" s="1" t="str">
-        <f t="shared" ca="1" si="6"/>
-        <v>Not necesary</v>
-      </c>
+      <c r="G33" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1620,16 +1688,105 @@
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Rejected">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Rejected">
       <formula>NOT(ISERROR(SEARCH("Rejected",E1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Not necesary">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Not necesary">
       <formula>NOT(ISERROR(SEARCH("Not necesary",G1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CFBD984-D573-43A4-B4C6-9DD0354D3D3A}">
+  <dimension ref="B1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="97.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="86.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="128" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="25.2" x14ac:dyDescent="0.5">
+      <c r="B1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+    </row>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F1">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Rejected">
+      <formula>NOT(ISERROR(SEARCH("Rejected",F1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Not necesary">
+      <formula>NOT(ISERROR(SEARCH("Not necesary",H1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
delete field's not necesary
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798522CE-78A7-438C-B774-5593237BFEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09642A09-8128-48E4-8C78-E0883362EF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="64">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -69,7 +69,10 @@
     <t>Approved</t>
   </si>
   <si>
-    <t>Imcomplete information</t>
+    <t>Bugget Exceeded</t>
+  </si>
+  <si>
+    <t>Not justified</t>
   </si>
   <si>
     <t>Request Type</t>
@@ -117,9 +120,6 @@
     <t>Rejected</t>
   </si>
   <si>
-    <t>Bugget</t>
-  </si>
-  <si>
     <t>REQ-002</t>
   </si>
   <si>
@@ -129,9 +129,6 @@
     <t>Supplies</t>
   </si>
   <si>
-    <t>Not necesary</t>
-  </si>
-  <si>
     <t>REQ-003</t>
   </si>
   <si>
@@ -229,6 +226,12 @@
   </si>
   <si>
     <t>REQ-030</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Incomplete information</t>
   </si>
 </sst>
 </file>
@@ -279,7 +282,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -326,24 +329,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -356,7 +346,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -912,25 +901,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="4">
         <v>46166</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F3" s="1">
         <v>21</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -941,10 +930,10 @@
         <v>46140</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>8</v>
@@ -953,12 +942,12 @@
         <v>16</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="4">
         <v>46121</v>
@@ -967,7 +956,7 @@
         <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>8</v>
@@ -976,18 +965,18 @@
         <v>12</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" s="4">
         <v>46137</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>28</v>
@@ -999,18 +988,18 @@
         <v>7</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="4">
         <v>46162</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>28</v>
@@ -1022,35 +1011,35 @@
         <v>35</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" s="4">
         <v>46144</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F8" s="1">
         <v>48</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B9" s="4">
         <v>46140</v>
@@ -1059,7 +1048,7 @@
         <v>27</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>8</v>
@@ -1068,21 +1057,21 @@
         <v>31</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B10" s="4">
         <v>46153</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>8</v>
@@ -1091,12 +1080,12 @@
         <v>24</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B11" s="4">
         <v>46141</v>
@@ -1105,21 +1094,21 @@
         <v>27</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F11" s="1">
         <v>23</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" s="4">
         <v>46164</v>
@@ -1137,21 +1126,21 @@
         <v>42</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B13" s="4">
         <v>46116</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>8</v>
@@ -1160,12 +1149,12 @@
         <v>18</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B14" s="4">
         <v>46125</v>
@@ -1177,64 +1166,64 @@
         <v>28</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F14" s="1">
         <v>5</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="4">
         <v>46143</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F15" s="1">
         <v>10</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="4">
         <v>46149</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F16" s="1">
         <v>14</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="4">
         <v>46125</v>
@@ -1243,7 +1232,7 @@
         <v>27</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>8</v>
@@ -1252,35 +1241,35 @@
         <v>9</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B18" s="4">
         <v>46142</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F18" s="1">
         <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B19" s="4">
         <v>46121</v>
@@ -1289,7 +1278,7 @@
         <v>27</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>8</v>
@@ -1298,21 +1287,21 @@
         <v>42</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B20" s="4">
         <v>46128</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>8</v>
@@ -1321,21 +1310,21 @@
         <v>18</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B21" s="4">
         <v>46152</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>8</v>
@@ -1344,12 +1333,12 @@
         <v>20</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B22" s="4">
         <v>46143</v>
@@ -1358,7 +1347,7 @@
         <v>27</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>8</v>
@@ -1367,21 +1356,21 @@
         <v>33</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B23" s="4">
         <v>46142</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>8</v>
@@ -1390,35 +1379,35 @@
         <v>18</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" s="4">
         <v>46156</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F24" s="1">
         <v>41</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B25" s="4">
         <v>46153</v>
@@ -1430,27 +1419,27 @@
         <v>28</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F25" s="1">
         <v>30</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B26" s="4">
         <v>46115</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>8</v>
@@ -1459,21 +1448,21 @@
         <v>46</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27" s="4">
         <v>46156</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>8</v>
@@ -1482,44 +1471,44 @@
         <v>6</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B28" s="4">
         <v>46133</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F28" s="1">
         <v>42</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>43</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B29" s="4">
         <v>46168</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>8</v>
@@ -1528,44 +1517,44 @@
         <v>14</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30" s="4">
         <v>46156</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F30" s="1">
         <v>16</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B31" s="4">
         <v>46157</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>8</v>
@@ -1573,36 +1562,36 @@
       <c r="F31" s="1">
         <v>27</v>
       </c>
-      <c r="G31" s="8" t="s">
-        <v>29</v>
+      <c r="G31" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B32" s="4">
         <v>46150</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F32" s="10">
+      <c r="F32" s="9">
         <v>26</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D33" s="5"/>
-      <c r="G33" s="9"/>
+      <c r="G33" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1640,7 +1629,7 @@
   <sheetData>
     <row r="1" spans="2:8" ht="25.2" x14ac:dyDescent="0.5">
       <c r="B1" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -1660,39 +1649,39 @@
         <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="C3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="11" t="s">
+      <c r="F3" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="G3" s="10" t="s">
         <v>20</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
now continued with dashboard - creating sheet dashboard
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09642A09-8128-48E4-8C78-E0883362EF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204F9D10-A654-4698-A233-F54029F4EF40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA" sheetId="1" r:id="rId1"/>
-    <sheet name="Excel Formula" sheetId="2" r:id="rId2"/>
+    <sheet name="Dashboard" sheetId="3" r:id="rId2"/>
+    <sheet name="Excel Formula" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -69,9 +70,6 @@
     <t>Approved</t>
   </si>
   <si>
-    <t>Bugget Exceeded</t>
-  </si>
-  <si>
     <t>Not justified</t>
   </si>
   <si>
@@ -135,9 +133,6 @@
     <t>REQ-004</t>
   </si>
   <si>
-    <t>Perssonel</t>
-  </si>
-  <si>
     <t>REQ-005</t>
   </si>
   <si>
@@ -232,6 +227,12 @@
   </si>
   <si>
     <t>Incomplete information</t>
+  </si>
+  <si>
+    <t>Personnel</t>
+  </si>
+  <si>
+    <t>Budget Exceeded</t>
   </si>
 </sst>
 </file>
@@ -901,39 +902,39 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" s="4">
         <v>46166</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F3" s="1">
         <v>21</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4">
         <v>46140</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>8</v>
@@ -942,21 +943,21 @@
         <v>16</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" s="4">
         <v>46121</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>8</v>
@@ -965,21 +966,21 @@
         <v>12</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4">
         <v>46137</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>8</v>
@@ -988,21 +989,21 @@
         <v>7</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B7" s="4">
         <v>46162</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>8</v>
@@ -1011,44 +1012,44 @@
         <v>35</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B8" s="4">
         <v>46144</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="F8" s="1">
         <v>48</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B9" s="4">
         <v>46140</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>8</v>
@@ -1057,21 +1058,21 @@
         <v>31</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B10" s="4">
         <v>46153</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>8</v>
@@ -1080,44 +1081,44 @@
         <v>24</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B11" s="4">
         <v>46141</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F11" s="1">
         <v>23</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B12" s="4">
         <v>46164</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>8</v>
@@ -1126,21 +1127,21 @@
         <v>42</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B13" s="4">
         <v>46116</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>8</v>
@@ -1149,90 +1150,90 @@
         <v>18</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B14" s="4">
         <v>46125</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="E14" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F14" s="1">
         <v>5</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B15" s="4">
         <v>46143</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F15" s="1">
         <v>10</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B16" s="4">
         <v>46149</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F16" s="1">
         <v>14</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B17" s="4">
         <v>46125</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>8</v>
@@ -1241,44 +1242,44 @@
         <v>9</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B18" s="4">
         <v>46142</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="F18" s="1">
         <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B19" s="4">
         <v>46121</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>8</v>
@@ -1287,21 +1288,21 @@
         <v>42</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B20" s="4">
         <v>46128</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>8</v>
@@ -1310,21 +1311,21 @@
         <v>18</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B21" s="4">
         <v>46152</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>8</v>
@@ -1333,21 +1334,21 @@
         <v>20</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B22" s="4">
         <v>46143</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>8</v>
@@ -1356,21 +1357,21 @@
         <v>33</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B23" s="4">
         <v>46142</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>8</v>
@@ -1379,67 +1380,67 @@
         <v>18</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B24" s="4">
         <v>46156</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F24" s="1">
         <v>41</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B25" s="4">
         <v>46153</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="E25" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F25" s="1">
         <v>30</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B26" s="4">
         <v>46115</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>8</v>
@@ -1448,21 +1449,21 @@
         <v>46</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B27" s="4">
         <v>46156</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>8</v>
@@ -1471,44 +1472,44 @@
         <v>6</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B28" s="4">
         <v>46133</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="F28" s="1">
         <v>42</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>9</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B29" s="4">
         <v>46168</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>8</v>
@@ -1517,44 +1518,44 @@
         <v>14</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B30" s="4">
         <v>46156</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F30" s="1">
         <v>16</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B31" s="4">
         <v>46157</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>8</v>
@@ -1563,21 +1564,21 @@
         <v>27</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B32" s="4">
         <v>46150</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>8</v>
@@ -1586,7 +1587,7 @@
         <v>26</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
@@ -1614,6 +1615,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3B0EF6E-767D-4F3A-831D-7BCA499C31E3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CFBD984-D573-43A4-B4C6-9DD0354D3D3A}">
   <dimension ref="B1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1629,7 +1639,7 @@
   <sheetData>
     <row r="1" spans="2:8" ht="25.2" x14ac:dyDescent="0.5">
       <c r="B1" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -1649,39 +1659,39 @@
         <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
         <v>5</v>
       </c>
       <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
         <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add KPIs in dashboARd sheet
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204F9D10-A654-4698-A233-F54029F4EF40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89CA8398-1E85-49A8-98DB-F069AC610BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="69">
   <si>
     <t xml:space="preserve">Dashboard KPIs </t>
   </si>
@@ -233,13 +233,31 @@
   </si>
   <si>
     <t>Budget Exceeded</t>
+  </si>
+  <si>
+    <t>Requirement Process - KPI Dashboard</t>
+  </si>
+  <si>
+    <t>Total request</t>
+  </si>
+  <si>
+    <t>Approval rate</t>
+  </si>
+  <si>
+    <t>Avg. Responde time (Hrs)</t>
+  </si>
+  <si>
+    <t>SLA compilance(&lt;24 hrs)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,6 +286,13 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -331,10 +356,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -350,11 +376,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="5">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -404,74 +434,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1616,9 +1578,72 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3B0EF6E-767D-4F3A-831D-7BCA499C31E3}">
-  <dimension ref="A1"/>
+  <dimension ref="B2:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="31.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4">
+        <f>COUNTA(DATA!A3:A32)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <f>COUNTIF(DATA!E3:E32,"Approved")</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <f>COUNTIF(DATA!E3:E32,"Rejected")</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="11">
+        <f>C5/C4</f>
+        <v>0.6333333333333333</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="12">
+        <f>AVERAGE(DATA!F3:F32)</f>
+        <v>23.533333333333335</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="13">
+        <f>COUNTIF(DATA!F3:F32,"&lt;=24")/Dashboard!C4</f>
+        <v>0.6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add auxiliar tabler - request by type
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84EB3102-942B-4E5F-9D59-10C632386952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D4F7FC-D318-4134-A45F-05FFCF09EDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="72">
   <si>
     <t>Request ID</t>
   </si>
@@ -247,13 +247,16 @@
     <t>SLA compliance(&lt;24 hrs)</t>
   </si>
   <si>
-    <t>Request by area</t>
-  </si>
-  <si>
     <t>Field operation</t>
   </si>
   <si>
     <t>Field Operations</t>
+  </si>
+  <si>
+    <t>Request by Area</t>
+  </si>
+  <si>
+    <t>Request by type</t>
   </si>
 </sst>
 </file>
@@ -372,7 +375,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -388,17 +391,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -881,7 +883,7 @@
         <v>46166</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>32</v>
@@ -950,7 +952,7 @@
         <v>46137</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>26</v>
@@ -1042,7 +1044,7 @@
         <v>46153</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>22</v>
@@ -1226,7 +1228,7 @@
         <v>46142</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>22</v>
@@ -1502,7 +1504,7 @@
         <v>46156</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>26</v>
@@ -1525,7 +1527,7 @@
         <v>46157</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>22</v>
@@ -1589,105 +1591,144 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3B0EF6E-767D-4F3A-831D-7BCA499C31E3}">
-  <dimension ref="B2:H9"/>
+  <dimension ref="B2:K9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="25.2" x14ac:dyDescent="0.5">
-      <c r="B2" s="14" t="s">
+    <row r="2" spans="2:11" ht="25.2" x14ac:dyDescent="0.5">
+      <c r="B2" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" s="16"/>
       <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+      <c r="H2" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="I2" s="16"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="E3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Field Operations")</f>
+        <v>6</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Materials")</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <f>COUNTA(DATA!A3:A32)</f>
         <v>30</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5">
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Logistics")</f>
+        <v>9</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Personnel")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1">
         <f>COUNTIF(DATA!E3:E32,"Approved")</f>
         <v>19</v>
       </c>
-      <c r="E5" t="s">
-        <v>69</v>
-      </c>
-      <c r="G5">
-        <f>COUNTIF(DATA!C3:C32,"Field Operations")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
+      <c r="E5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Packaging")</f>
+        <v>9</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Equipment")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <f>COUNTIF(DATA!E3:E32,"Rejected")</f>
         <v>11</v>
       </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6">
-        <f>COUNTIF(DATA!C3:C32,"Logistics")</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+      <c r="E6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Administration")</f>
+        <v>6</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Supplies")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C7" s="11">
         <f>C5/C4</f>
         <v>0.6333333333333333</v>
       </c>
-      <c r="E7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7">
-        <f>COUNTIF(DATA!C3:C32,"Packaging")</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B8" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C8" s="12">
         <f>AVERAGE(DATA!F3:F32)</f>
         <v>23.533333333333335</v>
       </c>
-      <c r="E8" t="s">
-        <v>30</v>
-      </c>
-      <c r="G8">
-        <f>COUNTIF(DATA!C3:C32,"Administration")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C9" s="13">
@@ -1696,10 +1737,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="E4:H4"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
creating graphic Approval Status - Rejected and Approved
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D4F7FC-D318-4134-A45F-05FFCF09EDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62670EEF-56BB-4D23-AF05-9702199F9B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -459,6 +459,911 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Approval Status</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-93E4-43D3-93A1-A709F36ACB12}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-93E4-43D3-93A1-A709F36ACB12}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-ES"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$B$5:$B$6</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Approved</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Rejected</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$C$5:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-93E4-43D3-93A1-A709F36ACB12}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="75"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>891540</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{854DFF97-0A57-99EA-C7A7-4BF251A26D14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1597,9 +2502,10 @@
     <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.44140625" customWidth="1"/>
+    <col min="7" max="7" width="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.6640625" customWidth="1"/>
     <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="2" bestFit="1" customWidth="1"/>
   </cols>
@@ -1738,6 +2644,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
creating bar chart request by area
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62670EEF-56BB-4D23-AF05-9702199F9B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1152537-5C4E-4F84-8E39-F2B0C2756BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -264,7 +264,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -375,32 +375,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -766,7 +765,436 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Request by</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-ES" baseline="0"/>
+              <a:t> Area</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-ES"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$E$3:$E$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Field operation</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Logistics</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Packaging</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Administration</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$F$3:$F$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E183-4617-8822-8D5C277E1E0B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="792886671"/>
+        <c:axId val="792886191"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="792886671"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-ES"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="792886191"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="792886191"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-ES"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="792886671"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:dTable>
+        <c:showHorzBorder val="1"/>
+        <c:showVertBorder val="1"/>
+        <c:showOutline val="1"/>
+        <c:showKeys val="1"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr rtl="0">
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+      </c:dTable>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1325,6 +1753,511 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1358,6 +2291,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>964766</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>172193</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>324686</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>172193</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95503744-E311-7F84-53E1-92383E8297FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1744,15 +2713,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.2" x14ac:dyDescent="0.5">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -2463,16 +3432,15 @@
       <c r="E32" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F32" s="9">
+      <c r="F32" s="6">
         <v>26</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D33" s="5"/>
-      <c r="G33" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2511,22 +3479,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="25.2" x14ac:dyDescent="0.5">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="16" t="s">
+      <c r="C2" s="13"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="F2" s="16"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="16" t="s">
+      <c r="F2" s="13"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="I2" s="16"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
@@ -2538,7 +3506,7 @@
         <f>COUNTIF(DATA!C3:C32,"Field Operations")</f>
         <v>6</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="14" t="s">
         <v>32</v>
       </c>
       <c r="I3" s="1">
@@ -2561,7 +3529,7 @@
         <f>COUNTIF(DATA!C3:C32,"Logistics")</f>
         <v>9</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="14" t="s">
         <v>60</v>
       </c>
       <c r="I4" s="1">
@@ -2584,7 +3552,7 @@
         <f>COUNTIF(DATA!C3:C32,"Packaging")</f>
         <v>9</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="14" t="s">
         <v>22</v>
       </c>
       <c r="I5" s="1">
@@ -2607,7 +3575,7 @@
         <f>COUNTIF(DATA!C3:C32,"Administration")</f>
         <v>6</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="14" t="s">
         <v>26</v>
       </c>
       <c r="I6" s="1">
@@ -2619,7 +3587,7 @@
       <c r="B7" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="8">
         <f>C5/C4</f>
         <v>0.6333333333333333</v>
       </c>
@@ -2628,7 +3596,7 @@
       <c r="B8" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="9">
         <f>AVERAGE(DATA!F3:F32)</f>
         <v>23.533333333333335</v>
       </c>
@@ -2637,7 +3605,7 @@
       <c r="B9" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="10">
         <f>COUNTIF(DATA!F3:F32,"&lt;=24")/Dashboard!C4</f>
         <v>0.6</v>
       </c>
@@ -2663,15 +3631,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="25.2" x14ac:dyDescent="0.5">
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
@@ -2697,25 +3665,25 @@
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="7" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
change color by indivudual barra
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1152537-5C4E-4F84-8E39-F2B0C2756BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A85D1C-93C9-4B87-A6D7-CF66DED36332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -859,6 +859,72 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-E183-4617-8822-8D5C277E1E0B}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-E183-4617-8822-8D5C277E1E0B}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-E183-4617-8822-8D5C277E1E0B}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:spPr>
               <a:noFill/>

</xml_diff>

<commit_message>
creating graphic bar chart request by type
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A85D1C-93C9-4B87-A6D7-CF66DED36332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78255D6-2831-4690-81D7-CC67B9364D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -800,13 +800,8 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-ES"/>
-              <a:t>Request by</a:t>
+              <a:t>Request  by area</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="es-ES" baseline="0"/>
-              <a:t> Area</a:t>
-            </a:r>
-            <a:endParaRPr lang="es-ES"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -926,62 +921,7 @@
             </c:extLst>
           </c:dPt>
           <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="es-ES"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
+            <c:delete val="1"/>
           </c:dLbls>
           <c:cat>
             <c:strRef>
@@ -1048,99 +988,12 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:title>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="es-ES"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="792886191"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="792886191"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="es-ES"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="792886671"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:dTable>
-        <c:showHorzBorder val="1"/>
-        <c:showVertBorder val="1"/>
-        <c:showOutline val="1"/>
-        <c:showKeys val="1"/>
         <c:spPr>
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -1155,10 +1008,10 @@
           <a:effectLst/>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
-            <a:pPr rtl="0">
+            <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
@@ -1174,7 +1027,400 @@
             <a:endParaRPr lang="es-ES"/>
           </a:p>
         </c:txPr>
-      </c:dTable>
+        <c:crossAx val="792886191"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="792886191"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="792886671"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Request  by type</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-ES"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$H$3:$H$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Materials</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Personnel</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Equipment</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Supplies</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$I$3:$I$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-A064-4D0D-B5C3-47178B349D3A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="792886671"/>
+        <c:axId val="792886191"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="792886671"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="792886191"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="792886191"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="792886671"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -1300,6 +1546,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
@@ -1820,6 +2106,511 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2393,6 +3184,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>436756</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>317067</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC9F03FC-3D40-42AA-B529-BEDF6858B7B1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>

<commit_message>
ending fase 3 with dashboard kpis and excel graphics
</commit_message>
<xml_diff>
--- a/Dashboard/DashboardKPIs.xlsx
+++ b/Dashboard/DashboardKPIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User_Job\Documents\Bizagi\Field requirement Management\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78255D6-2831-4690-81D7-CC67B9364D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D0E9215-B75E-48DF-8E63-383F3B5FBDDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BFDDE99E-5C7D-432D-B837-4C5E5869A86E}"/>
   </bookViews>
@@ -925,7 +925,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$E$3:$E$6</c:f>
+              <c:f>Dashboard!$B$18:$B$21</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -945,7 +945,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$F$3:$F$6</c:f>
+              <c:f>Dashboard!$C$18:$C$21</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1270,7 +1270,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$H$3:$H$6</c:f>
+              <c:f>Dashboard!$B$32:$B$35</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1290,7 +1290,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$I$3:$I$6</c:f>
+              <c:f>Dashboard!$C$32:$C$35</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -3119,16 +3119,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>135673</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>152864</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>891540</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>399585</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>176561</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3155,16 +3155,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>964766</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>172193</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>109838</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>88559</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>324686</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>172193</xdr:rowOff>
+      <xdr:colOff>371706</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>157975</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3191,16 +3191,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>436756</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>120806</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>167268</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>317067</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>362415</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>74342</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4359,11 +4359,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3B0EF6E-767D-4F3A-831D-7BCA499C31E3}">
-  <dimension ref="B2:K9"/>
+  <dimension ref="B2:O35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.44140625" customWidth="1"/>
     <col min="7" max="7" width="2" bestFit="1" customWidth="1"/>
@@ -4371,45 +4371,27 @@
     <col min="9" max="9" width="5.6640625" customWidth="1"/>
     <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="32.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="25.2" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:15" ht="25.2" x14ac:dyDescent="0.5">
       <c r="B2" s="13" t="s">
         <v>65</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="11"/>
-      <c r="E2" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F2" s="13"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="I2" s="13"/>
       <c r="J2" s="12"/>
       <c r="K2" s="12"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="O2" s="12"/>
+    </row>
+    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="E3" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F3" s="1">
-        <f>COUNTIF(DATA!C3:C32,"Field Operations")</f>
-        <v>6</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="I3" s="1">
-        <f>COUNTIF(DATA!D3:D32,"Materials")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>62</v>
       </c>
@@ -4417,22 +4399,8 @@
         <f>COUNTA(DATA!A3:A32)</f>
         <v>30</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="1">
-        <f>COUNTIF(DATA!C3:C32,"Logistics")</f>
-        <v>9</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="I4" s="1">
-        <f>COUNTIF(DATA!D3:D32,"Personnel")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
@@ -4440,22 +4408,8 @@
         <f>COUNTIF(DATA!E3:E32,"Approved")</f>
         <v>19</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="1">
-        <f>COUNTIF(DATA!C3:C32,"Packaging")</f>
-        <v>9</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="1">
-        <f>COUNTIF(DATA!D3:D32,"Equipment")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>23</v>
       </c>
@@ -4463,22 +4417,8 @@
         <f>COUNTIF(DATA!E3:E32,"Rejected")</f>
         <v>11</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="1">
-        <f>COUNTIF(DATA!C3:C32,"Administration")</f>
-        <v>6</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="1">
-        <f>COUNTIF(DATA!D3:D32,"Supplies")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>63</v>
       </c>
@@ -4487,7 +4427,7 @@
         <v>0.6333333333333333</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>66</v>
       </c>
@@ -4496,13 +4436,97 @@
         <v>23.533333333333335</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C9" s="10">
         <f>COUNTIF(DATA!F3:F32,"&lt;=24")/Dashboard!C4</f>
         <v>0.6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" ht="25.2" x14ac:dyDescent="0.5">
+      <c r="B17" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="13"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B18" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Field Operations")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Logistics")</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Packaging")</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B21" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="1">
+        <f>COUNTIF(DATA!C3:C32,"Administration")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" ht="25.2" x14ac:dyDescent="0.5">
+      <c r="B31" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="13"/>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B32" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Materials")</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B33" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Personnel")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B34" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C34" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Equipment")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B35" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" s="1">
+        <f>COUNTIF(DATA!D3:D32,"Supplies")</f>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>